<commit_message>
- add example based on excel file in package
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="35">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -116,6 +116,18 @@
   </si>
   <si>
     <t xml:space="preserve">x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">doesn’t work yet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#IF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q1 == 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">abc = 7</t>
   </si>
 </sst>
 </file>
@@ -149,12 +161,18 @@
       <family val="0"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -191,8 +209,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -214,56 +240,56 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="10.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="0" t="s">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>12</v>
       </c>
     </row>
@@ -284,337 +310,337 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="0" t="n">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="0" t="n">
+      <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="0" t="n">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C4" s="0" t="s">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="0" t="n">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="0" t="n">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="0" t="n">
+      <c r="A7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="1" t="n">
         <v>99</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C13" s="0" t="s">
+      <c r="B13" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="0" t="n">
+      <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="0" t="n">
+      <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C19" s="0" t="s">
+      <c r="B19" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="0" t="n">
+      <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C23" s="0" t="s">
+      <c r="C23" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B24" s="0" t="n">
+      <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C24" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B25" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C25" s="0" t="s">
+      <c r="B25" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B26" s="0" t="n">
+      <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C26" s="0" t="s">
+      <c r="C26" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B27" s="0" t="n">
+      <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="C27" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="0" t="n">
+      <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="C28" s="1" t="s">
         <v>26</v>
       </c>
     </row>
@@ -635,7 +661,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -652,18 +678,32 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultColWidth="10.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultColWidth="10.70703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="0" t="n">
+      <c r="C1" s="1" t="n">
         <v>1</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F2" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
change excel mapping code
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="40">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -118,9 +118,6 @@
     <t xml:space="preserve">x</t>
   </si>
   <si>
-    <t xml:space="preserve">doesn’t work yet</t>
-  </si>
-  <si>
     <t xml:space="preserve">#IF</t>
   </si>
   <si>
@@ -133,7 +130,7 @@
     <t xml:space="preserve">#REC</t>
   </si>
   <si>
-    <t xml:space="preserve">kq2</t>
+    <t xml:space="preserve">kq3</t>
   </si>
   <si>
     <t xml:space="preserve">summarized variable</t>
@@ -188,8 +185,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -258,7 +255,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -328,7 +325,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -679,7 +676,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -696,10 +693,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="10.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -709,78 +706,76 @@
       <c r="C1" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F2" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="1" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="B5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="0" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="0" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="C7" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" s="0" t="n">
-        <v>2</v>
-      </c>
-      <c r="E7" s="0" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="B8" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="B8" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="C8" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="D8" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" s="0" t="s">
-        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add 1st version of #KG creating multiple variables
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="41">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -143,6 +143,9 @@
   </si>
   <si>
     <t xml:space="preserve">4-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#KG</t>
   </si>
 </sst>
 </file>
@@ -255,7 +258,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -325,7 +328,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -676,7 +679,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -693,8 +696,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -776,6 +779,17 @@
       </c>
       <c r="E8" s="1" t="s">
         <v>39</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- repair #VARL - add example to xlsx
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="44">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -146,6 +146,15 @@
   </si>
   <si>
     <t xml:space="preserve">#KG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#VARL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">my new label</t>
   </si>
 </sst>
 </file>
@@ -696,7 +705,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -790,6 +799,28 @@
       </c>
       <c r="C10" s="0" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
repair #VALL and add example to excel
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="49">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -155,6 +155,21 @@
   </si>
   <si>
     <t xml:space="preserve">my new label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#VALL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">overwrite new label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">also with</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value labels </t>
+  </si>
+  <si>
+    <t xml:space="preserve">now</t>
   </si>
 </sst>
 </file>
@@ -164,7 +179,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -186,6 +201,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -236,7 +257,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -246,6 +267,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -705,7 +730,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -821,6 +846,44 @@
       </c>
       <c r="C12" s="0" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="0" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
repair #AVALL and add example to excel
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="51">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -170,6 +170,12 @@
   </si>
   <si>
     <t xml:space="preserve">now</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#AVALL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">added label</t>
   </si>
 </sst>
 </file>
@@ -730,7 +736,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -884,6 +890,25 @@
       </c>
       <c r="C17" s="3" t="s">
         <v>48</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- took the file write_verbatims7.R from K:\Tools\R\write_verbatims and modified it to make it run - added verbatim sheet in mapping.xlsx - add the file Verbatims_fake survey_20201204UW.xlsx to the package included files folder; this file was generated in the project K:\Projects\UW fake survey
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" state="visible" r:id="rId2"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="91">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -40,12 +40,18 @@
     <t xml:space="preserve">How much do you like the product?</t>
   </si>
   <si>
+    <t xml:space="preserve">Like Product</t>
+  </si>
+  <si>
     <t xml:space="preserve">q2</t>
   </si>
   <si>
     <t xml:space="preserve">Do you want to recommend the product?</t>
   </si>
   <si>
+    <t xml:space="preserve">recommend product</t>
+  </si>
+  <si>
     <t xml:space="preserve">q3</t>
   </si>
   <si>
@@ -64,6 +70,9 @@
     <t xml:space="preserve">How much do you like your best friend?</t>
   </si>
   <si>
+    <t xml:space="preserve">Like best friend</t>
+  </si>
+  <si>
     <t xml:space="preserve">nv</t>
   </si>
   <si>
@@ -97,9 +106,15 @@
     <t xml:space="preserve">normal</t>
   </si>
   <si>
+    <t xml:space="preserve">bbb</t>
+  </si>
+  <si>
     <t xml:space="preserve">much</t>
   </si>
   <si>
+    <t xml:space="preserve">ccc</t>
+  </si>
+  <si>
     <t xml:space="preserve">very much</t>
   </si>
   <si>
@@ -110,6 +125,111 @@
   </si>
   <si>
     <t xml:space="preserve">no</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verbatims file</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daten\10_MergeFiles.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID-Variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DC_ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID-Format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replace</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filename result</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K:\Projects\UW fake survey\Verbatims\Verbatims_fake survey_20201204.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filename input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">K:\Projects\UW fake survey\Verbatims\Verbatims_fake survey_20201204UW.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read from line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read to line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VariableOriginal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EFA1MCG2MDG3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tabellen-blatt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nebeneinander?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VariableOriginal_umbenannt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VarOrigMissing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VariableZiel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VariableZähler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VariableLabel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VariableMissing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max.Codestufen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CodestufenLabel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reserved</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max.Zuordnungen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BisherigerWertAnzeigen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WeitereVariablen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Titel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q6n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q7n</t>
   </si>
   <si>
     <t xml:space="preserve">#COMP</t>
@@ -318,37 +438,46 @@
       <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="C2" s="0" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -375,25 +504,25 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -404,16 +533,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -424,7 +553,10 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="G3" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -435,7 +567,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
+      </c>
+      <c r="G4" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="0" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -446,7 +584,13 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
+      </c>
+      <c r="G5" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="0" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -457,7 +601,10 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
+      </c>
+      <c r="G6" s="0" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -468,238 +615,238 @@
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -718,9 +865,165 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+  <dimension ref="B1:R1048576"/>
+  <sheetFormatPr defaultColWidth="10.6875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B1" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B2" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B3" s="0" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="0" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="D9" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="0" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>48</v>
+      </c>
+      <c r="E15" s="0" t="s">
+        <v>49</v>
+      </c>
+      <c r="F15" s="0" t="s">
+        <v>50</v>
+      </c>
+      <c r="G15" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="H15" s="0" t="s">
+        <v>52</v>
+      </c>
+      <c r="I15" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="J15" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="K15" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="L15" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="M15" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="N15" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="O15" s="0" t="s">
+        <v>59</v>
+      </c>
+      <c r="P15" s="0" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q15" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="R15" s="0" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="H16" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="R16" s="0" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="H17" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="R17" s="0" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L18" s="0" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="L19" s="0" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+  </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -741,10 +1044,10 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="C1" s="1" t="n">
         <v>1</v>
@@ -753,27 +1056,27 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>31</v>
+        <v>71</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>32</v>
+        <v>72</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>35</v>
+        <v>75</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>36</v>
+        <v>76</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -787,7 +1090,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>37</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -806,7 +1109,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>38</v>
+        <v>78</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>4</v>
@@ -818,15 +1121,15 @@
         <v>3</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>39</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10" s="0" t="s">
         <v>3</v>
@@ -834,10 +1137,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>29</v>
+        <v>69</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>41</v>
+        <v>81</v>
       </c>
       <c r="C11" s="0" t="n">
         <v>1</v>
@@ -845,24 +1148,24 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>41</v>
+        <v>81</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>43</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>41</v>
+        <v>81</v>
       </c>
       <c r="C14" s="0" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -870,7 +1173,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>46</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -878,37 +1181,37 @@
         <v>2</v>
       </c>
       <c r="C16" s="0" t="s">
-        <v>47</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>38</v>
+        <v>78</v>
       </c>
       <c r="B17" s="0" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>48</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>49</v>
+        <v>89</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>41</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>38</v>
+        <v>78</v>
       </c>
       <c r="B20" s="0" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="0" t="s">
-        <v>50</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
- add free2 - now the commands are executed according to the sequence of sheets in the mapping file
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="Labels" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="Verbatims" sheetId="3" state="visible" r:id="rId4"/>
     <sheet name="Free1" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="Free2" sheetId="5" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="94">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -302,6 +303,9 @@
   </si>
   <si>
     <t xml:space="preserve">added label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">free2_var</t>
   </si>
 </sst>
 </file>
@@ -1242,4 +1246,34 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A2:C2"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>93</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
use relative path from mapping file path root
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" state="visible" r:id="rId2"/>
@@ -155,7 +155,7 @@
     <t xml:space="preserve">Filename input</t>
   </si>
   <si>
-    <t xml:space="preserve">inst/extdata/Verbatims_fake_survey.xlsx</t>
+    <t xml:space="preserve">Verbatims_fake_survey.xlsx</t>
   </si>
   <si>
     <t xml:space="preserve">Read from line</t>
@@ -430,7 +430,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -509,7 +509,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -878,7 +878,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:R1048576"/>
-  <sheetFormatPr defaultColWidth="10.7421875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1052,7 +1052,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1254,16 +1254,16 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add mdg & mcg test example
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="98">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -231,6 +231,18 @@
   </si>
   <si>
     <t xml:space="preserve">q7n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q6mdg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q6_{nn}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q6mcg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q6n{nn}</t>
   </si>
   <si>
     <t xml:space="preserve">#COMP</t>
@@ -430,7 +442,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.82421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -509,7 +521,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.82421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -878,7 +890,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:R1048576"/>
-  <sheetFormatPr defaultColWidth="10.75" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.76953125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1023,11 +1035,35 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="H18" s="0" t="s">
+        <v>70</v>
+      </c>
       <c r="L18" s="1" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="0" t="s">
+        <v>63</v>
+      </c>
+      <c r="C19" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="H19" s="0" t="s">
+        <v>72</v>
+      </c>
       <c r="L19" s="1" t="n">
         <v>100</v>
       </c>
@@ -1052,14 +1088,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.82421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C1" s="1" t="n">
         <v>1</v>
@@ -1068,38 +1104,38 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1113,7 +1149,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1132,7 +1168,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>4</v>
@@ -1144,12 +1180,12 @@
         <v>3</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>6</v>
@@ -1160,10 +1196,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>1</v>
@@ -1171,24 +1207,24 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1196,7 +1232,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1204,37 +1240,37 @@
         <v>2</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -1254,14 +1290,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
skip 16 lines (and add two lines to sheet in mapping file as in new version)
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -442,7 +442,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultColWidth="10.83984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -521,7 +521,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.83984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -890,7 +890,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:R1048576"/>
-  <sheetFormatPr defaultColWidth="10.78515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -947,91 +947,57 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E15" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="F15" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="I15" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="J15" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="K15" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="L15" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="M15" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="N15" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="O15" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="P15" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="Q15" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="R15" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="R16" s="1" t="s">
-        <v>64</v>
-      </c>
-    </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="C17" s="1" t="n">
-        <v>1</v>
+        <v>46</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>47</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>67</v>
+        <v>48</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>51</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>68</v>
+        <v>52</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="M17" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="N17" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="P17" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q17" s="1" t="s">
+        <v>61</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1039,37 +1005,69 @@
         <v>63</v>
       </c>
       <c r="C18" s="1" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="L18" s="1" t="n">
-        <v>100</v>
+        <v>65</v>
+      </c>
+      <c r="R18" s="1" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C19" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="R19" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="C19" s="1" t="n">
+      <c r="C20" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="L20" s="1" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C21" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D21" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="H21" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="L19" s="1" t="n">
+      <c r="L21" s="1" t="n">
         <v>100</v>
       </c>
     </row>
-    <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1088,7 +1086,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F20"/>
-  <sheetFormatPr defaultColWidth="10.83984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1290,7 +1288,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">

</xml_diff>

<commit_message>
replace single equals signs to double equals signs for: - second column for #IF - third columns for #COMP - and add these examples to mapping
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Variables" sheetId="1" state="visible" r:id="rId2"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="99">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -251,10 +251,13 @@
     <t xml:space="preserve">x</t>
   </si>
   <si>
+    <t xml:space="preserve">q1 = 2</t>
+  </si>
+  <si>
     <t xml:space="preserve">#IF</t>
   </si>
   <si>
-    <t xml:space="preserve">q1 == 1</t>
+    <t xml:space="preserve">q1 = 1</t>
   </si>
   <si>
     <t xml:space="preserve">abc = 7</t>
@@ -1095,45 +1098,45 @@
       <c r="B1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="C1" s="1" t="n">
-        <v>1</v>
+      <c r="C1" s="1" t="s">
+        <v>75</v>
       </c>
       <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1147,7 +1150,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1166,7 +1169,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>4</v>
@@ -1178,12 +1181,12 @@
         <v>3</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>6</v>
@@ -1197,7 +1200,7 @@
         <v>73</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>1</v>
@@ -1205,24 +1208,24 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>87</v>
-      </c>
       <c r="C12" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1230,7 +1233,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1238,37 +1241,37 @@
         <v>2</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -1295,7 +1298,7 @@
         <v>73</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add Operation and `New var name` columns in "Variables" sheet
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="102">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -35,6 +35,12 @@
     <t xml:space="preserve">new_label</t>
   </si>
   <si>
+    <t xml:space="preserve">op</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new_name</t>
+  </si>
+  <si>
     <t xml:space="preserve">q1</t>
   </si>
   <si>
@@ -63,6 +69,9 @@
   </si>
   <si>
     <t xml:space="preserve">How much do you like your friends?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q4_renamed</t>
   </si>
   <si>
     <t xml:space="preserve">q5</t>
@@ -444,10 +453,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -457,54 +466,63 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -531,56 +549,56 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -588,47 +606,47 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -636,244 +654,244 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -897,49 +915,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -947,108 +965,108 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C20" s="1" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="L20" s="1" t="n">
         <v>100</v>
@@ -1056,16 +1074,16 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C21" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="L21" s="1" t="n">
         <v>100</v>
@@ -1088,55 +1106,55 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1150,7 +1168,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1169,7 +1187,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>4</v>
@@ -1181,26 +1199,26 @@
         <v>3</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>1</v>
@@ -1208,24 +1226,24 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B14" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>88</v>
-      </c>
       <c r="C14" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1233,7 +1251,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1241,39 +1259,43 @@
         <v>2</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -1295,10 +1317,10 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add rename() command for Variables sheet
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="103">
   <si>
     <t xml:space="preserve">var</t>
   </si>
@@ -59,6 +59,9 @@
     <t xml:space="preserve">recommend product</t>
   </si>
   <si>
+    <t xml:space="preserve">q2_renamed</t>
+  </si>
+  <si>
     <t xml:space="preserve">q3</t>
   </si>
   <si>
@@ -272,7 +275,7 @@
     <t xml:space="preserve">abc = 7</t>
   </si>
   <si>
-    <t xml:space="preserve">q{2 3} == 1</t>
+    <t xml:space="preserve">q{2_renamed 3} == 1</t>
   </si>
   <si>
     <t xml:space="preserve">kq{5 6} = {7 8}</t>
@@ -339,7 +342,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -369,6 +372,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -419,7 +429,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -433,6 +443,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -454,7 +468,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -466,10 +480,10 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
@@ -484,7 +498,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -494,35 +508,38 @@
       <c r="C3" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="E3" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="E5" s="0" t="s">
         <v>15</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -542,32 +559,32 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -578,16 +595,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -598,7 +615,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -612,13 +629,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -629,13 +646,13 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -646,7 +663,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -660,7 +677,7 @@
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -671,7 +688,7 @@
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -682,7 +699,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -693,205 +710,205 @@
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -911,53 +928,53 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:R1048576"/>
-  <sheetFormatPr defaultColWidth="10.796875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -965,108 +982,108 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H18" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="R18" s="1" t="s">
         <v>68</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H19" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="R19" s="1" t="s">
         <v>71</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C20" s="1" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="L20" s="1" t="n">
         <v>100</v>
@@ -1074,16 +1091,16 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C21" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L21" s="1" t="n">
         <v>100</v>
@@ -1107,54 +1124,54 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F26"/>
-  <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1168,7 +1185,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1187,7 +1204,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>4</v>
@@ -1199,15 +1216,15 @@
         <v>3</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>8</v>
+        <v>91</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>5</v>
@@ -1215,10 +1232,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>1</v>
@@ -1226,24 +1243,24 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>91</v>
-      </c>
       <c r="C12" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1251,7 +1268,7 @@
         <v>1</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1259,37 +1276,37 @@
         <v>2</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1313,14 +1330,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
remove #KG command from mapping as it breaks with rename(). However, it should be refactored anyway!
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -381,7 +381,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -392,6 +392,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -429,7 +435,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -446,7 +452,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1123,7 +1133,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1220,13 +1230,13 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="H10" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="I10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="J10" s="4" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
small modifications I can't remember
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="116">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -355,6 +355,9 @@
   </si>
   <si>
     <t xml:space="preserve">Almost same variable label for q{3 5} and q{5 3}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">should be ignored</t>
   </si>
   <si>
     <t xml:space="preserve">a{1 2}</t>
@@ -379,7 +382,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -416,6 +419,14 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -472,7 +483,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -494,6 +505,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1233,7 +1248,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1432,27 +1447,38 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="B25" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C26" s="6" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="B25" s="0" t="s">
-        <v>110</v>
-      </c>
-      <c r="C25" s="0" t="s">
+      <c r="B27" s="0" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="C27" s="0" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="B26" s="0" t="s">
-        <v>112</v>
-      </c>
-      <c r="C26" s="0" t="s">
+      <c r="B28" s="0" t="s">
         <v>113</v>
       </c>
-    </row>
+      <c r="C28" s="0" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -1477,7 +1503,7 @@
         <v>83</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
also replace multiple single equal signs in e.g. in condition statements with OR or AND
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -288,7 +288,7 @@
     <t xml:space="preserve">#IF</t>
   </si>
   <si>
-    <t xml:space="preserve">q1 = 1</t>
+    <t xml:space="preserve">q1 = 1 | q3 = 2</t>
   </si>
   <si>
     <t xml:space="preserve">abc = 7</t>
@@ -382,7 +382,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -412,13 +412,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <u val="single"/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -504,11 +497,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -530,21 +523,21 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
@@ -565,7 +558,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.90234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -656,7 +649,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.90234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1025,7 +1018,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:R22"/>
-  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.83984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1248,237 +1241,249 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J30"/>
-  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:J32"/>
+  <sheetFormatPr defaultColWidth="10.90234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="F1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B3" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="F1" s="3"/>
-    </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B4" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B5" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="1" t="n">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="1" t="n">
+      <c r="C8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="1" t="n">
+      <c r="D8" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="1" t="n">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="1" t="n">
+      <c r="C9" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="1" t="n">
+      <c r="E9" s="1" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="1" t="n">
+      <c r="B10" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="1" t="n">
+      <c r="C10" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D8" s="1" t="n">
+      <c r="D10" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H10" s="4" t="s">
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H12" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I12" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="J10" s="4" t="s">
+      <c r="J12" s="4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="C11" s="1" t="n">
+      <c r="C13" s="1" t="n">
         <v>1</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>98</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C16" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="1" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="1" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C18" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B17" s="1" t="n">
+      <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B21" s="1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B20" s="1" t="n">
+      <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C22" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C24" s="0" t="s">
+      <c r="C26" s="1" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="6" t="s">
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="6" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C26" s="6" t="s">
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C28" s="6" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C27" s="0" t="s">
+      <c r="C29" s="1" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B30" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C28" s="0" t="s">
+      <c r="C30" s="1" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -1496,7 +1501,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">

</xml_diff>

<commit_message>
add small Value section in function help
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="117">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -325,6 +325,9 @@
   </si>
   <si>
     <t xml:space="preserve">#VARL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n </t>
   </si>
   <si>
     <t xml:space="preserve">my new label</t>
@@ -1376,21 +1379,21 @@
         <v>99</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>98</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1398,7 +1401,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1406,7 +1409,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1417,12 +1420,13 @@
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>105</v>
-      </c>
-    </row>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>98</v>
@@ -1436,7 +1440,7 @@
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1445,20 +1449,20 @@
         <v>99</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1466,10 +1470,10 @@
         <v>83</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1477,10 +1481,10 @@
         <v>99</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -1508,7 +1512,7 @@
         <v>83</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add function for #DIC
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="118">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -373,6 +373,9 @@
   </si>
   <si>
     <t xml:space="preserve">same variable label for a1 &amp; a2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#DIC</t>
   </si>
   <si>
     <t xml:space="preserve">free2_var</t>
@@ -1487,7 +1490,17 @@
         <v>115</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="s">
+        <v>116</v>
+      </c>
+      <c r="B32" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -1512,7 +1525,7 @@
         <v>83</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
perhaps 1st version of working severalize also for multiline command blocks
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="121">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -303,7 +303,10 @@
     <t xml:space="preserve">#REC</t>
   </si>
   <si>
-    <t xml:space="preserve">kq3</t>
+    <t xml:space="preserve">q{1 3}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kq{1 3}</t>
   </si>
   <si>
     <t xml:space="preserve">summarized variable</t>
@@ -376,6 +379,12 @@
   </si>
   <si>
     <t xml:space="preserve">#DIC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">r_expr_var</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ifelse(q1 == 5, q3 * 10, q1 * 8) %&gt;% haven::labelled(label = “varlab”)</t>
   </si>
   <si>
     <t xml:space="preserve">free2_var</t>
@@ -1247,7 +1256,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr defaultColWidth="10.90234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1296,18 +1305,18 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>91</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>16</v>
+        <v>92</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1321,7 +1330,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1340,7 +1349,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1352,12 +1361,12 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H12" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I12" s="5" t="s">
         <v>15</v>
@@ -1371,7 +1380,7 @@
         <v>83</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1379,24 +1388,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1404,7 +1413,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1412,60 +1421,60 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1473,32 +1482,40 @@
         <v>83</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B32" s="0" t="s">
         <v>16</v>
       </c>
       <c r="C32" s="0" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="0" t="s">
+        <v>118</v>
+      </c>
+      <c r="C34" s="0" t="s">
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -1525,7 +1542,7 @@
         <v>83</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
fix bug: derive severalize index for columns 2 to 4 not only column 2 of free sheet
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="122">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -379,6 +379,9 @@
   </si>
   <si>
     <t xml:space="preserve">#DIC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q{2 4}_renamed</t>
   </si>
   <si>
     <t xml:space="preserve">r_expr_var</t>
@@ -1507,15 +1510,15 @@
         <v>16</v>
       </c>
       <c r="C32" s="0" t="s">
-        <v>15</v>
+        <v>118</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="0" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C34" s="0" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
   </sheetData>
@@ -1542,7 +1545,7 @@
         <v>83</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add #COMPR (like #COMP but without replacement of single equal signs in column 3)
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="125">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -384,10 +384,19 @@
     <t xml:space="preserve">q{2 4}_renamed</t>
   </si>
   <si>
+    <t xml:space="preserve">!!! Standard auto-correction in libre-office changes quote style:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">see here: https://superuser.com/a/643521</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#COMPR</t>
+  </si>
+  <si>
     <t xml:space="preserve">r_expr_var</t>
   </si>
   <si>
-    <t xml:space="preserve">ifelse(q1 == 5, q3 * 10, q1 * 8) %&gt;% haven::labelled(label = “varlab”)</t>
+    <t xml:space="preserve">ifelse(q1 == 5, q3 * 10, q1 * 8) %&gt;% haven::labelled(label = "varlab")</t>
   </si>
   <si>
     <t xml:space="preserve">free2_var</t>
@@ -494,7 +503,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -523,6 +532,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1259,7 +1272,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J34"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr defaultColWidth="10.90234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1513,15 +1526,31 @@
         <v>118</v>
       </c>
     </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C33" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="0" t="s">
-        <v>119</v>
-      </c>
-      <c r="C34" s="0" t="s">
+      <c r="C34" s="7" t="s">
         <v>120</v>
       </c>
     </row>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="0" t="s">
+        <v>121</v>
+      </c>
+      <c r="B35" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="C35" s="0" t="s">
+        <v>123</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C34" r:id="rId1" display="https://superuser.com/a/643521"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
   <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1545,7 +1574,7 @@
         <v>83</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add #RFUN command block
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="131">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -406,6 +406,15 @@
   </si>
   <si>
     <t xml:space="preserve">q1 q2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#RFUN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/home/chief/R/datenanpassr/inst/extdata/example_R_function.R</t>
+  </si>
+  <si>
+    <t xml:space="preserve">create_string_var</t>
   </si>
   <si>
     <t xml:space="preserve">free2_var</t>
@@ -1281,7 +1290,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J39"/>
   <sheetFormatPr defaultColWidth="10.90234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1568,6 +1577,17 @@
       </c>
       <c r="D37" s="0" t="s">
         <v>126</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>128</v>
+      </c>
+      <c r="C39" s="0" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -1597,7 +1617,7 @@
         <v>83</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
put #KG back in Excel file
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -544,11 +544,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -578,7 +578,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -613,7 +613,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="10.90234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -704,7 +704,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.90234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1073,7 +1073,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:R22"/>
-  <sheetFormatPr defaultColWidth="10.83984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1296,8 +1296,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
-  <sheetFormatPr defaultColWidth="10.90234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F41"/>
+  <sheetFormatPr defaultColWidth="10.921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1405,14 +1405,14 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H12" s="4" t="s">
+      <c r="A12" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="B12" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="J12" s="4" t="s">
-        <v>9</v>
+      <c r="C12" s="4" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1540,13 +1540,13 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="B32" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C32" s="0" t="s">
+      <c r="C32" s="1" t="s">
         <v>118</v>
       </c>
     </row>
@@ -1561,52 +1561,52 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B35" s="0" t="s">
+      <c r="B35" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C35" s="0" t="s">
+      <c r="C35" s="1" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+      <c r="A37" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B37" s="0" t="s">
+      <c r="B37" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="C37" s="0" t="s">
+      <c r="C37" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D37" s="0" t="s">
+      <c r="D37" s="1" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
+      <c r="A39" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="B39" s="0" t="s">
+      <c r="B39" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="C39" s="0" t="s">
+      <c r="C39" s="1" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
+      <c r="A41" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B41" s="0" t="s">
+      <c r="B41" s="1" t="s">
         <v>131</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C34" r:id="rId1" display="https://superuser.com/a/643521"/>
+    <hyperlink ref="C34" r:id="rId1" display="see here: https://superuser.com/a/643521"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
@@ -1624,7 +1624,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">

</xml_diff>

<commit_message>
decide by config variable whether to execute "Label" sheet before "Variables" sheet
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="134">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -37,6 +37,9 @@
   </si>
   <si>
     <t xml:space="preserve">id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Excecute before variable sheet?</t>
   </si>
   <si>
     <t xml:space="preserve">var</t>
@@ -430,8 +433,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -527,12 +531,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -577,7 +585,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -594,6 +602,14 @@
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -617,74 +633,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>
@@ -708,59 +724,59 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -768,47 +784,47 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -816,244 +832,244 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1077,49 +1093,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1127,154 +1143,154 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H18" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="R18" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H19" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="R19" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="R19" s="1" t="s">
-        <v>75</v>
-      </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C20" s="2" t="n">
+      <c r="B20" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D20" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2" t="s">
+      <c r="D20" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="I20" s="2"/>
-      <c r="J20" s="2"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2" t="n">
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C21" s="2" t="n">
+      <c r="B21" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D21" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="E21" s="2"/>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2" t="n">
+      <c r="D21" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1303,60 +1319,60 @@
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="F1" s="3"/>
+      <c r="F1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="F2" s="3"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="3"/>
+        <v>86</v>
+      </c>
+      <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>88</v>
       </c>
+      <c r="C4" s="3" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="A5" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>90</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1370,7 +1386,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1389,7 +1405,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1401,26 +1417,26 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>92</v>
+      <c r="A12" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1428,24 +1444,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1453,7 +1469,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1461,147 +1477,147 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="6" t="s">
-        <v>112</v>
+      <c r="B27" s="7" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="6" t="s">
-        <v>112</v>
+      <c r="C28" s="7" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="7" t="s">
-        <v>119</v>
+      <c r="C33" s="8" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="7" t="s">
-        <v>120</v>
+      <c r="C34" s="8" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -1628,10 +1644,10 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add command block function set_na_to_filter_except()
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="138">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -42,6 +42,21 @@
     <t xml:space="preserve">Excecute before variable sheet?</t>
   </si>
   <si>
+    <t xml:space="preserve">variables not recoded to FILTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">missing values recoded to</t>
+  </si>
+  <si>
+    <t xml:space="preserve">missing values labelled by</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FILTER</t>
+  </si>
+  <si>
     <t xml:space="preserve">var</t>
   </si>
   <si>
@@ -55,9 +70,6 @@
   </si>
   <si>
     <t xml:space="preserve">new_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">q1</t>
   </si>
   <si>
     <t xml:space="preserve">How much do you like the product?</t>
@@ -585,7 +597,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -610,6 +622,30 @@
       </c>
       <c r="B3" s="2" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -633,74 +669,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -724,59 +760,59 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -784,47 +820,47 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -832,244 +868,244 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>
@@ -1093,49 +1129,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1143,111 +1179,111 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1258,19 +1294,19 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1281,16 +1317,16 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1329,50 +1365,50 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1386,7 +1422,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1405,7 +1441,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1417,26 +1453,26 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1444,24 +1480,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>100</v>
-      </c>
       <c r="C16" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1469,7 +1505,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1477,147 +1513,147 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="7" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="7" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="8" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="8" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1644,10 +1680,10 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add possibility to manipulate command table in config
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="142">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -57,6 +57,15 @@
     <t xml:space="preserve">FILTER</t>
   </si>
   <si>
+    <t xml:space="preserve">manipulate command table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">df_cmd %&gt;% dplyr::filter(TRUE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(does nothing, but by changing the filter argument, can be used to filter the list of commands)</t>
+  </si>
+  <si>
     <t xml:space="preserve">var</t>
   </si>
   <si>
@@ -253,6 +262,9 @@
   </si>
   <si>
     <t xml:space="preserve">Titel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DONT</t>
   </si>
   <si>
     <t xml:space="preserve">q6</t>
@@ -597,7 +609,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -646,6 +658,17 @@
       </c>
       <c r="B6" s="0" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -669,19 +692,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -689,54 +712,54 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -760,28 +783,28 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -792,16 +815,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -812,7 +835,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -826,13 +849,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -843,13 +866,13 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -860,7 +883,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -874,238 +897,238 @@
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -1124,54 +1147,54 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:R22"/>
+  <dimension ref="B1:S22"/>
   <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1179,111 +1202,114 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>75</v>
+        <v>78</v>
+      </c>
+      <c r="S17" s="0" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1294,19 +1320,19 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1317,16 +1343,16 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1365,50 +1391,50 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1422,7 +1448,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1441,7 +1467,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1453,26 +1479,26 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1480,24 +1506,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>104</v>
-      </c>
       <c r="C16" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1505,7 +1531,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1513,147 +1539,147 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="7" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="7" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="8" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="8" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -1680,10 +1706,10 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add comments column title in "configr" sheet, to prevent New names: * `` -> ...3
message....
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,12 +25,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="143">
   <si>
     <t xml:space="preserve">item</t>
   </si>
   <si>
     <t xml:space="preserve">value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comments</t>
   </si>
   <si>
     <t xml:space="preserve">id_var</t>
@@ -619,18 +622,21 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="0" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" s="2" t="b">
         <v>1</v>
@@ -638,15 +644,15 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="0" t="n">
         <v>-2</v>
@@ -654,21 +660,21 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" s="0" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -692,74 +698,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -783,59 +789,59 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -843,47 +849,47 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -891,244 +897,244 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1152,49 +1158,49 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1202,114 +1208,114 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="S17" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H18" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="R18" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H19" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="R19" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1320,19 +1326,19 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1343,16 +1349,16 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1391,50 +1397,50 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1448,7 +1454,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1467,7 +1473,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1479,26 +1485,26 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1506,24 +1512,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1531,7 +1537,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1539,147 +1545,147 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="8" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
   </sheetData>
@@ -1706,10 +1712,10 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
use keyword "yes" instead of "TRUE" because otherwise we might mix things up between German and English versions of Excel (readxl imports the Excel boolean TRUE as "1", so let's choose something more stable...)
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="143">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -45,6 +45,9 @@
     <t xml:space="preserve">Excecute before variable sheet?</t>
   </si>
   <si>
+    <t xml:space="preserve">yes</t>
+  </si>
+  <si>
     <t xml:space="preserve">variables not recoded to FILTER</t>
   </si>
   <si>
@@ -174,9 +177,6 @@
     <t xml:space="preserve">no answer</t>
   </si>
   <si>
-    <t xml:space="preserve">yes</t>
-  </si>
-  <si>
     <t xml:space="preserve">no</t>
   </si>
   <si>
@@ -441,7 +441,7 @@
     <t xml:space="preserve">#RFUN</t>
   </si>
   <si>
-    <t xml:space="preserve">/home/chief/R/datenanpassr/inst/extdata/example_R_function.R</t>
+    <t xml:space="preserve">example_R_function.R</t>
   </si>
   <si>
     <t xml:space="preserve">calc_sum_of_k_vars</t>
@@ -558,7 +558,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -567,7 +567,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -576,14 +576,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -612,8 +604,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -622,7 +614,7 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -635,48 +627,49 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="b">
-        <v>1</v>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="0" t="n">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="n">
         <v>-2</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="B6" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
+      <c r="C7" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -694,78 +687,78 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="10.921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.94140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -785,63 +778,63 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.94140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -849,47 +842,47 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -897,29 +890,29 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>49</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2</v>
@@ -930,211 +923,211 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1154,7 +1147,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="10.859375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1263,7 +1256,7 @@
       <c r="R17" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="S17" s="0" t="s">
+      <c r="S17" s="1" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1381,7 +1374,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F41"/>
-  <sheetFormatPr defaultColWidth="10.921875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.94140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1489,13 +1482,13 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B12" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="5" t="s">
+      <c r="B12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>102</v>
       </c>
     </row>
@@ -1559,7 +1552,6 @@
         <v>117</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
         <v>118</v>
@@ -1592,12 +1584,12 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="5" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="7" t="s">
+      <c r="C28" s="5" t="s">
         <v>122</v>
       </c>
     </row>
@@ -1628,19 +1620,19 @@
         <v>127</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="6" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="6" t="s">
         <v>130</v>
       </c>
     </row>
@@ -1708,7 +1700,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">

</xml_diff>

<commit_message>
add possibility to modify value label by "new label" column on "Label" sheet
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="143">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -177,6 +177,9 @@
     <t xml:space="preserve">no answer</t>
   </si>
   <si>
+    <t xml:space="preserve">YES</t>
+  </si>
+  <si>
     <t xml:space="preserve">no</t>
   </si>
   <si>
@@ -409,9 +412,6 @@
   </si>
   <si>
     <t xml:space="preserve">#DIC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">q{2 4}_renamed</t>
   </si>
   <si>
     <t xml:space="preserve">!!! Standard auto-correction in libre-office changes quote style:</t>
@@ -605,7 +605,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -687,7 +687,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="10.94140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.95703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -778,7 +778,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.94140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.95703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -888,7 +888,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -909,6 +909,9 @@
       <c r="C8" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="E8" s="0" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
@@ -918,7 +921,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1147,53 +1150,53 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="10.8671875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1201,114 +1204,114 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H18" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="R18" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H19" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="R19" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1319,19 +1322,19 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1342,16 +1345,16 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1374,7 +1377,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F41"/>
-  <sheetFormatPr defaultColWidth="10.94140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.95703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1390,50 +1393,50 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1447,7 +1450,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1466,7 +1469,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1478,26 +1481,26 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>25</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1505,24 +1508,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1530,7 +1533,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1538,92 +1541,92 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>128</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1700,11 +1703,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>142</v>

</xml_diff>

<commit_message>
if nothing in configr field "variables not recoded to FILTER" then return empty vector, not NA
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="143">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -51,40 +51,40 @@
     <t xml:space="preserve">variables not recoded to FILTER</t>
   </si>
   <si>
+    <t xml:space="preserve">missing values recoded to</t>
+  </si>
+  <si>
+    <t xml:space="preserve">missing values labelled by</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FILTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">manipulate command table</t>
+  </si>
+  <si>
+    <t xml:space="preserve">df_cmd %&gt;% dplyr::filter(TRUE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(does nothing, but by changing the filter argument, can be used to filter the list of commands)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">var</t>
+  </si>
+  <si>
+    <t xml:space="preserve">varlab</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new_label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">op</t>
+  </si>
+  <si>
+    <t xml:space="preserve">new_name</t>
+  </si>
+  <si>
     <t xml:space="preserve">q1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">missing values recoded to</t>
-  </si>
-  <si>
-    <t xml:space="preserve">missing values labelled by</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FILTER</t>
-  </si>
-  <si>
-    <t xml:space="preserve">manipulate command table</t>
-  </si>
-  <si>
-    <t xml:space="preserve">df_cmd %&gt;% dplyr::filter(TRUE)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(does nothing, but by changing the filter argument, can be used to filter the list of commands)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">var</t>
-  </si>
-  <si>
-    <t xml:space="preserve">varlab</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new_label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">op</t>
-  </si>
-  <si>
-    <t xml:space="preserve">new_name</t>
   </si>
   <si>
     <t xml:space="preserve">How much do you like the product?</t>
@@ -634,17 +634,15 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>8</v>
-      </c>
+      <c r="B4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>-2</v>
@@ -652,21 +650,21 @@
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -691,24 +689,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>18</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>20</v>
@@ -782,7 +780,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>34</v>
@@ -794,7 +792,7 @@
         <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>37</v>
@@ -808,7 +806,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
@@ -828,7 +826,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
@@ -842,7 +840,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
@@ -859,7 +857,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
@@ -876,7 +874,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
@@ -890,7 +888,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>99</v>

</xml_diff>

<commit_message>
define added id column variable name in configr sheet
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="144">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -42,6 +42,12 @@
     <t xml:space="preserve">id</t>
   </si>
   <si>
+    <t xml:space="preserve">added id variable name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DC_ID</t>
+  </si>
+  <si>
     <t xml:space="preserve">Excecute before variable sheet?</t>
   </si>
   <si>
@@ -190,9 +196,6 @@
   </si>
   <si>
     <t xml:space="preserve">ID-Variable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DC_ID</t>
   </si>
   <si>
     <t xml:space="preserve">ID-Format</t>
@@ -604,8 +607,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
-  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -630,7 +633,7 @@
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
     </row>
@@ -638,36 +641,44 @@
       <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>-2</v>
-      </c>
+        <v>9</v>
+      </c>
+      <c r="B5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="1" t="n">
+        <v>-2</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="1" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="B8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -685,78 +696,78 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="10.95703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.9765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -776,63 +787,63 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.95703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.9765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -840,47 +851,47 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -888,247 +899,247 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="0" t="s">
-        <v>50</v>
+        <v>8</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1148,53 +1159,53 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.90234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>55</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1202,114 +1213,114 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H18" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="R18" s="1" t="s">
         <v>84</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H19" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="R19" s="1" t="s">
         <v>87</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1320,19 +1331,19 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1343,16 +1354,16 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1375,7 +1386,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F41"/>
-  <sheetFormatPr defaultColWidth="10.95703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.9765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1391,50 +1402,50 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1448,7 +1459,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1467,7 +1478,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1479,26 +1490,26 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1506,24 +1517,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1531,7 +1542,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1539,146 +1550,146 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -1701,14 +1712,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
also allow  #REC for recoding to new values by providing multiple lines mapping on the same new value and taking the new value label from the first line
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="149">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -454,6 +454,21 @@
   </si>
   <si>
     <t xml:space="preserve">df %&gt;% dplyr::mutate(a=1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q1  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">kkq1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b</t>
   </si>
   <si>
     <t xml:space="preserve">free2_var</t>
@@ -608,7 +623,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -696,7 +711,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="10.9765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -787,7 +802,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.9765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1159,7 +1174,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="10.90234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.921875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1385,8 +1400,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
-  <sheetFormatPr defaultColWidth="10.9765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F49"/>
+  <sheetFormatPr defaultColWidth="10.984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1690,6 +1705,66 @@
       </c>
       <c r="B41" s="1" t="s">
         <v>142</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="0" t="s">
+        <v>103</v>
+      </c>
+      <c r="B44" s="0" t="s">
+        <v>143</v>
+      </c>
+      <c r="C44" s="0" t="s">
+        <v>144</v>
+      </c>
+      <c r="D44" s="0" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E45" s="0" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D46" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="E46" s="0" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D47" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B48" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D48" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B49" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D49" s="0" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1712,14 +1787,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>95</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add autorecode option to variable sheet
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="149">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -135,6 +135,12 @@
     <t xml:space="preserve">Like best friend</t>
   </si>
   <si>
+    <t xml:space="preserve">q6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a</t>
+  </si>
+  <si>
     <t xml:space="preserve">nv</t>
   </si>
   <si>
@@ -276,9 +282,6 @@
     <t xml:space="preserve">DONT</t>
   </si>
   <si>
-    <t xml:space="preserve">q6</t>
-  </si>
-  <si>
     <t xml:space="preserve">Q6</t>
   </si>
   <si>
@@ -463,9 +466,6 @@
   </si>
   <si>
     <t xml:space="preserve">vl</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a</t>
   </si>
   <si>
     <t xml:space="preserve">b</t>
@@ -623,7 +623,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.66796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -710,8 +710,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="10.984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -783,6 +783,14 @@
       </c>
       <c r="C6" s="1" t="s">
         <v>35</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -802,32 +810,32 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="10.984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -838,16 +846,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -858,7 +866,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -872,13 +880,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -889,13 +897,13 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -906,7 +914,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -920,7 +928,7 @@
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -934,7 +942,7 @@
         <v>8</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -945,7 +953,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -956,7 +964,7 @@
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -967,7 +975,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -978,7 +986,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -989,7 +997,7 @@
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1000,7 +1008,7 @@
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1011,7 +1019,7 @@
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1022,7 +1030,7 @@
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1033,7 +1041,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1044,7 +1052,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1055,7 +1063,7 @@
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1066,7 +1074,7 @@
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1077,7 +1085,7 @@
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1088,7 +1096,7 @@
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1099,7 +1107,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1110,7 +1118,7 @@
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1121,7 +1129,7 @@
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1132,7 +1140,7 @@
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1143,7 +1151,7 @@
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1154,7 +1162,7 @@
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -1174,19 +1182,19 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="10.921875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.94140625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -1194,33 +1202,33 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1228,114 +1236,114 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H18" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="R18" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H19" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="R19" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1346,19 +1354,19 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1369,16 +1377,16 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1401,7 +1409,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="10.984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1417,50 +1425,50 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1474,7 +1482,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1493,7 +1501,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1505,26 +1513,26 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>27</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1532,24 +1540,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1557,7 +1565,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1565,86 +1573,86 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>28</v>
@@ -1655,115 +1663,115 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
-        <v>103</v>
-      </c>
-      <c r="B44" s="0" t="s">
-        <v>143</v>
-      </c>
-      <c r="C44" s="0" t="s">
+      <c r="A44" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B44" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="D44" s="0" t="s">
+      <c r="C44" s="1" t="s">
         <v>145</v>
       </c>
+      <c r="D44" s="1" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="0" t="n">
+      <c r="B45" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D45" s="0" t="n">
+      <c r="D45" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="E45" s="0" t="s">
-        <v>146</v>
+      <c r="E45" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="0" t="n">
+      <c r="B46" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D46" s="0" t="n">
+      <c r="D46" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="E46" s="0" t="s">
+      <c r="E46" s="1" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="0" t="n">
+      <c r="B47" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D47" s="0" t="n">
+      <c r="D47" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="0" t="n">
+      <c r="B48" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D48" s="0" t="n">
+      <c r="D48" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="0" t="n">
+      <c r="B49" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D49" s="0" t="n">
+      <c r="D49" s="1" t="n">
         <v>2</v>
       </c>
     </row>
@@ -1787,11 +1795,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>148</v>

</xml_diff>

<commit_message>
adapt tests for #KG
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="150">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -361,6 +361,9 @@
   </si>
   <si>
     <t xml:space="preserve">#KG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kq1</t>
   </si>
   <si>
     <t xml:space="preserve">n</t>
@@ -1520,11 +1523,11 @@
       <c r="A12" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1532,7 +1535,7 @@
         <v>96</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1540,24 +1543,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1565,7 +1568,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1573,7 +1576,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1584,15 +1587,15 @@
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1603,29 +1606,29 @@
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1633,26 +1636,26 @@
         <v>96</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>28</v>
@@ -1663,56 +1666,56 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1720,13 +1723,13 @@
         <v>104</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1748,7 +1751,7 @@
         <v>2</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1802,7 +1805,7 @@
         <v>96</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add string to numeric variable transformation from "Variables" sheet
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="153">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -141,6 +141,18 @@
     <t xml:space="preserve">a</t>
   </si>
   <si>
+    <t xml:space="preserve">q8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A numeric variable in string format.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Now the variable is in numeric format.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n</t>
+  </si>
+  <si>
     <t xml:space="preserve">nv</t>
   </si>
   <si>
@@ -364,9 +376,6 @@
   </si>
   <si>
     <t xml:space="preserve">kq1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n</t>
   </si>
   <si>
     <t xml:space="preserve">#VARL</t>
@@ -626,7 +635,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.6875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -713,8 +722,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultColWidth="11.01953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr defaultColWidth="11.0390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -794,6 +803,20 @@
       </c>
       <c r="D7" s="1" t="s">
         <v>37</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>39</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -813,32 +836,32 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="11.01953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.0390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -849,16 +872,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -869,7 +892,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -883,13 +906,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -900,13 +923,13 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -917,7 +940,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -931,7 +954,7 @@
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -945,7 +968,7 @@
         <v>8</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -956,7 +979,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -967,7 +990,7 @@
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -978,7 +1001,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -989,7 +1012,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1000,7 +1023,7 @@
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1011,7 +1034,7 @@
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1022,7 +1045,7 @@
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1033,7 +1056,7 @@
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1044,7 +1067,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1055,7 +1078,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1066,7 +1089,7 @@
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1077,7 +1100,7 @@
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1088,7 +1111,7 @@
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1099,7 +1122,7 @@
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1110,7 +1133,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1121,7 +1144,7 @@
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1132,7 +1155,7 @@
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1143,7 +1166,7 @@
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1154,7 +1177,7 @@
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1165,7 +1188,7 @@
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1185,19 +1208,19 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="10.95703125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.9765625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -1205,33 +1228,33 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1239,63 +1262,63 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1306,30 +1329,30 @@
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1340,13 +1363,13 @@
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1357,19 +1380,19 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1386,10 +1409,10 @@
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1412,7 +1435,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="11.01953125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.0390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1428,50 +1451,50 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1485,7 +1508,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1504,7 +1527,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1516,15 +1539,15 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>27</v>
@@ -1532,10 +1555,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>113</v>
+        <v>41</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1543,24 +1566,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>113</v>
+        <v>41</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1568,7 +1591,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1576,86 +1599,86 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>113</v>
+        <v>41</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="5" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>28</v>
@@ -1666,70 +1689,70 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="6" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="6" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1751,7 +1774,7 @@
         <v>2</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1798,14 +1821,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add drop variables dataset transformation from "Variables" sheet
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="155">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -151,6 +151,12 @@
   </si>
   <si>
     <t xml:space="preserve">n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d</t>
   </si>
   <si>
     <t xml:space="preserve">nv</t>
@@ -722,7 +728,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultColWidth="11.0390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -817,6 +823,14 @@
       </c>
       <c r="D8" s="0" t="s">
         <v>41</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -843,25 +857,25 @@
         <v>16</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -872,16 +886,16 @@
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -892,7 +906,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -906,13 +920,13 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -923,13 +937,13 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -940,7 +954,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -954,7 +968,7 @@
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -968,7 +982,7 @@
         <v>8</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -979,7 +993,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -990,7 +1004,7 @@
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1001,7 +1015,7 @@
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1012,7 +1026,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1023,7 +1037,7 @@
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1034,7 +1048,7 @@
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1045,7 +1059,7 @@
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1056,7 +1070,7 @@
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1067,7 +1081,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1078,7 +1092,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1089,7 +1103,7 @@
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1100,7 +1114,7 @@
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1111,7 +1125,7 @@
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1122,7 +1136,7 @@
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1133,7 +1147,7 @@
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1144,7 +1158,7 @@
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1155,7 +1169,7 @@
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1166,7 +1180,7 @@
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1177,7 +1191,7 @@
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1188,7 +1202,7 @@
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1212,15 +1226,15 @@
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -1228,33 +1242,33 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1262,63 +1276,63 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1329,30 +1343,30 @@
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1363,13 +1377,13 @@
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1380,19 +1394,19 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1409,10 +1423,10 @@
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1451,50 +1465,50 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1508,7 +1522,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1527,7 +1541,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1539,15 +1553,15 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>27</v>
@@ -1555,7 +1569,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>41</v>
@@ -1566,24 +1580,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1591,7 +1605,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1599,23 +1613,23 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>41</v>
@@ -1623,62 +1637,62 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>28</v>
@@ -1689,70 +1703,70 @@
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1774,7 +1788,7 @@
         <v>2</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1825,10 +1839,10 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
- write results of mapp_configr() to variables in datenanpassr.env package environment - change wording in "configr" sheet
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="159">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -42,37 +42,67 @@
     <t xml:space="preserve">id</t>
   </si>
   <si>
-    <t xml:space="preserve">added id variable name</t>
+    <t xml:space="preserve">added_id_var</t>
   </si>
   <si>
     <t xml:space="preserve">DC_ID</t>
   </si>
   <si>
-    <t xml:space="preserve">Excecute before variable sheet?</t>
+    <t xml:space="preserve">Another id variable is added to the dataset. Choose the name of this variable here.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lab_before_var_sheet</t>
   </si>
   <si>
     <t xml:space="preserve">yes</t>
   </si>
   <si>
-    <t xml:space="preserve">variables not recoded to FILTER</t>
+    <t xml:space="preserve">If "yes", the commands on the "Label" sheet are excecuted before those of the "Variables" sheet.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">not_miss_to_filter_vars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Space-separated list of variable names, where the missing value is not recoded to FILTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">miss_rec_val</t>
   </si>
   <si>
     <t xml:space="preserve">missing values recoded to</t>
   </si>
   <si>
-    <t xml:space="preserve">missing values labelled by</t>
+    <t xml:space="preserve">miss_rec_lab</t>
   </si>
   <si>
     <t xml:space="preserve">FILTER</t>
   </si>
   <si>
-    <t xml:space="preserve">manipulate command table</t>
+    <t xml:space="preserve">manipulate_command_table</t>
   </si>
   <si>
     <t xml:space="preserve">df_cmd %&gt;% dplyr::filter(TRUE)</t>
   </si>
   <si>
-    <t xml:space="preserve">(does nothing, but by changing the filter argument, can be used to filter the list of commands)</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">manipulate command table; </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(does nothing, but by changing the filter argument (TRUE), can be used to filter the list of commands)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">var</t>
@@ -500,7 +530,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -522,6 +552,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <u val="single"/>
@@ -594,7 +630,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -603,11 +639,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -615,7 +655,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -641,7 +681,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.70703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -669,46 +709,58 @@
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="2" t="s">
         <v>8</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B5" s="1"/>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>-2</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C6" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
@@ -729,108 +781,108 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.0390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.0546875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>39</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>41</v>
+      <c r="A8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>42</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>43</v>
+      <c r="A9" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
   </sheetData>
@@ -850,63 +902,63 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="11.0390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.0546875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G3" s="1" t="n">
         <v>1</v>
@@ -914,47 +966,47 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G4" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G5" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="G6" s="1" t="n">
         <v>3</v>
@@ -962,247 +1014,247 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1222,19 +1274,19 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="10.9765625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -1242,33 +1294,33 @@
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1276,157 +1328,157 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C20" s="3" t="n">
+      <c r="B20" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3" t="n">
+      <c r="D20" s="4" t="s">
         <v>100</v>
       </c>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="I20" s="4"/>
+      <c r="J20" s="4"/>
+      <c r="K20" s="4"/>
+      <c r="L20" s="4" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C21" s="3" t="n">
+      <c r="B21" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C21" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="D21" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3" t="n">
+      <c r="D21" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="I21" s="4"/>
+      <c r="J21" s="4"/>
+      <c r="K21" s="4"/>
+      <c r="L21" s="4" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1449,66 +1501,66 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="11.0390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.0546875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="F1" s="4"/>
+      <c r="F1" s="5"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="F2" s="4"/>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="F3" s="4"/>
+        <v>108</v>
+      </c>
+      <c r="F3" s="5"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>107</v>
+      <c r="A4" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="A5" s="4" t="s">
         <v>109</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1522,7 +1574,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1541,7 +1593,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1553,26 +1605,26 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1580,24 +1632,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1605,7 +1657,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1613,160 +1665,160 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="5" t="s">
-        <v>131</v>
+      <c r="B27" s="6" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="5" t="s">
-        <v>131</v>
+      <c r="C28" s="6" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="6" t="s">
-        <v>137</v>
+      <c r="C33" s="7" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="6" t="s">
-        <v>138</v>
+      <c r="C34" s="7" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1777,7 +1829,7 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1788,7 +1840,7 @@
         <v>2</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1835,14 +1887,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.8046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add #SUMVAR (summary variable from Label sheet) - adapt Excel mapping file (created summary variable was overwritten by #REC on Free1...)
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -84,25 +84,7 @@
     <t xml:space="preserve">df_cmd %&gt;% dplyr::filter(TRUE)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">manipulate command table; </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(does nothing, but by changing the filter argument (TRUE), can be used to filter the list of commands)</t>
-    </r>
+    <t xml:space="preserve">manipulate command table; (does nothing, but by changing the filter argument (TRUE), can be used to filter the list of commands)</t>
   </si>
   <si>
     <t xml:space="preserve">var</t>
@@ -210,37 +192,37 @@
     <t xml:space="preserve">not at all</t>
   </si>
   <si>
+    <t xml:space="preserve">a bit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">much</t>
+  </si>
+  <si>
+    <t xml:space="preserve">very much</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no answer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no</t>
+  </si>
+  <si>
     <t xml:space="preserve">test</t>
   </si>
   <si>
     <t xml:space="preserve">aaa</t>
   </si>
   <si>
-    <t xml:space="preserve">a bit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">normal</t>
-  </si>
-  <si>
     <t xml:space="preserve">bbb</t>
   </si>
   <si>
-    <t xml:space="preserve">much</t>
-  </si>
-  <si>
     <t xml:space="preserve">ccc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">very much</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no answer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">YES</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no</t>
   </si>
   <si>
     <t xml:space="preserve">Verbatims file</t>
@@ -530,7 +512,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -552,12 +534,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <u val="single"/>
@@ -630,7 +606,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -639,15 +615,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -655,7 +627,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -681,7 +653,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -709,7 +681,7 @@
       <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
     </row>
@@ -717,7 +689,7 @@
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -759,7 +731,7 @@
       <c r="B8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>19</v>
       </c>
     </row>
@@ -781,7 +753,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.0546875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.07421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -902,7 +874,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="11.0546875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.07421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -930,7 +902,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
@@ -940,17 +912,11 @@
       <c r="C2" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="G2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>25</v>
       </c>
@@ -958,13 +924,11 @@
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="G3" s="1" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>55</v>
+      </c>
+      <c r="G3" s="1"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
         <v>25</v>
       </c>
@@ -972,16 +936,12 @@
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>56</v>
+      </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
         <v>25</v>
       </c>
@@ -989,16 +949,12 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="G5" s="1" t="n">
-        <v>3</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>57</v>
+      </c>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
         <v>25</v>
       </c>
@@ -1006,11 +962,9 @@
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="G6" s="1" t="n">
-        <v>3</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="G6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
@@ -1020,7 +974,7 @@
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1034,7 +988,7 @@
         <v>9</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1045,7 +999,7 @@
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1056,7 +1010,7 @@
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1078,7 +1032,7 @@
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1089,7 +1043,7 @@
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1100,7 +1054,7 @@
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1111,7 +1065,7 @@
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1122,7 +1076,7 @@
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1144,7 +1098,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1155,7 +1109,7 @@
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1166,7 +1120,7 @@
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1177,7 +1131,7 @@
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1188,10 +1142,10 @@
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
         <v>37</v>
       </c>
@@ -1201,8 +1155,17 @@
       <c r="C23" s="1" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F23" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="G23" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
         <v>37</v>
       </c>
@@ -1210,10 +1173,13 @@
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>55</v>
+      </c>
+      <c r="G24" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
         <v>37</v>
       </c>
@@ -1221,10 +1187,16 @@
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>56</v>
+      </c>
+      <c r="G25" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
         <v>37</v>
       </c>
@@ -1232,10 +1204,16 @@
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>57</v>
+      </c>
+      <c r="G26" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
         <v>37</v>
       </c>
@@ -1243,7 +1221,10 @@
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
+      </c>
+      <c r="G27" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1254,7 +1235,7 @@
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1274,7 +1255,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="10.984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1422,48 +1403,48 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="4" t="s">
+      <c r="B20" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="4" t="n">
+      <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4" t="s">
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4" t="n">
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="C21" s="4" t="n">
+      <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4" t="s">
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4" t="n">
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3" t="n">
         <v>100</v>
       </c>
     </row>
@@ -1501,19 +1482,19 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="11.0546875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.07421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="F1" s="5"/>
+      <c r="F1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-      <c r="F2" s="5"/>
+      <c r="F2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
@@ -1525,27 +1506,27 @@
       <c r="C3" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="F3" s="5"/>
+      <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1711,12 +1692,12 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="5" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="5" t="s">
         <v>135</v>
       </c>
     </row>
@@ -1754,12 +1735,12 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="6" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="6" t="s">
         <v>142</v>
       </c>
     </row>
@@ -1887,7 +1868,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.8046875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">

</xml_diff>

<commit_message>
- add #RECNA method - add #COMPR method - modify #COMPR command block in excel file not to use pipe - export `[.command_blocks`
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -462,7 +462,35 @@
     <t xml:space="preserve">r_expr_var</t>
   </si>
   <si>
-    <t xml:space="preserve">ifelse(q1 == 5, q3 * 10, q1 * 8) %&gt;% haven::labelled(label = "varlab")</t>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">haven::labelled(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ifelse(q1 == 5, q3 * 10, q1 * 8), </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">label = "varlab")</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">#MERGE</t>
@@ -512,7 +540,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -550,6 +578,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -653,7 +687,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="11.7421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -753,7 +787,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.07421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.09375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -874,7 +908,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="11.07421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.09375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1255,7 +1289,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="11.00390625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.01953125" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1482,7 +1516,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="11.07421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.09375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1868,7 +1902,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">

</xml_diff>

<commit_message>
remove replacing single equal sign functionality
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -352,13 +352,13 @@
     <t xml:space="preserve">x</t>
   </si>
   <si>
-    <t xml:space="preserve">q1 = 2</t>
+    <t xml:space="preserve">q1 == 2</t>
   </si>
   <si>
     <t xml:space="preserve">#IF</t>
   </si>
   <si>
-    <t xml:space="preserve">q1 = 1 | q3 = 2</t>
+    <t xml:space="preserve">q1 == 1 | q3 == 2</t>
   </si>
   <si>
     <t xml:space="preserve">abc = 7</t>
@@ -654,7 +654,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11.72265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -742,7 +742,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.15625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.19140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -863,7 +863,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="11.15625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.19140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1244,7 +1244,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="11.01171875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.0390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1471,7 +1471,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="11.15625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.19140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1856,7 +1856,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">

</xml_diff>

<commit_message>
fill named region R_not_miss_to_filter_vars in Excel mapping file (resulting in parameter not_miss_to_filter_vars)
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="158">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -59,6 +59,9 @@
   </si>
   <si>
     <t xml:space="preserve">not_miss_to_filter_vars</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q1 q5</t>
   </si>
   <si>
     <t xml:space="preserve">Space-separated list of variable names, where the missing value is not recoded to FILTER</t>
@@ -654,7 +657,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11.7578125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -690,39 +693,41 @@
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="1"/>
+      <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
       <c r="C4" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>-2</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -742,108 +747,108 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.19140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -863,43 +868,43 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="11.19140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -907,68 +912,68 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
@@ -977,192 +982,192 @@
         <v>6</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G24" s="1" t="n">
         <v>1</v>
@@ -1170,47 +1175,47 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G25" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="G26" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G27" s="1" t="n">
         <v>3</v>
@@ -1218,13 +1223,13 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>
@@ -1244,53 +1249,53 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="11.0390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.0546875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1298,114 +1303,114 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H18" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="R18" s="1" t="s">
         <v>94</v>
-      </c>
-      <c r="R18" s="1" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H19" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="R19" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1416,19 +1421,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1439,16 +1444,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1471,7 +1476,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="11.19140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1487,50 +1492,50 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1544,7 +1549,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1563,7 +1568,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1575,26 +1580,26 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1602,24 +1607,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1627,7 +1632,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1635,159 +1640,159 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1798,7 +1803,7 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1809,7 +1814,7 @@
         <v>2</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1856,14 +1861,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.9140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
add further column "further_ex_cond" to table in Excel mapping "Verbatims" sheet: allowing to specify additional condition whether to copy the verbatim values to the data
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="159">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -313,13 +313,16 @@
     <t xml:space="preserve">Titel</t>
   </si>
   <si>
-    <t xml:space="preserve">DONT</t>
+    <t xml:space="preserve">further_ex_cond</t>
   </si>
   <si>
     <t xml:space="preserve">Q6</t>
   </si>
   <si>
     <t xml:space="preserve">q6n</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q5 != 1</t>
   </si>
   <si>
     <t xml:space="preserve">q7</t>
@@ -657,7 +660,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11.77734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -747,7 +750,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.2109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -868,7 +871,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="11.2109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1249,7 +1252,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="11.0546875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.07421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1378,22 +1381,25 @@
       <c r="R18" s="1" t="s">
         <v>94</v>
       </c>
+      <c r="S18" s="0" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H19" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="R19" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1404,13 +1410,13 @@
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1421,19 +1427,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1450,10 +1456,10 @@
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
@@ -1476,7 +1482,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="11.2109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.2265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1492,50 +1498,50 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1549,7 +1555,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1568,7 +1574,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1580,15 +1586,15 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>29</v>
@@ -1596,7 +1602,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>43</v>
@@ -1607,24 +1613,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1632,7 +1638,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1640,23 +1646,23 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>43</v>
@@ -1664,61 +1670,61 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>30</v>
@@ -1729,70 +1735,70 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1814,7 +1820,7 @@
         <v>2</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1861,14 +1867,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.9296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
rename argument further_ex_cond to ex_further_cond
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -313,7 +313,7 @@
     <t xml:space="preserve">Titel</t>
   </si>
   <si>
-    <t xml:space="preserve">further_ex_cond</t>
+    <t xml:space="preserve">ex_further_cond</t>
   </si>
   <si>
     <t xml:space="preserve">Q6</t>
@@ -660,7 +660,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11.78515625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.8046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -750,7 +750,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.2265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -871,7 +871,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="11.2265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1252,7 +1252,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="11.07421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.09375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1309,7 +1309,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
         <v>76</v>
       </c>
@@ -1381,7 +1381,7 @@
       <c r="R18" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="S18" s="0" t="s">
+      <c r="S18" s="1" t="s">
         <v>96</v>
       </c>
     </row>
@@ -1482,7 +1482,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="11.2265625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1867,7 +1867,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.94140625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.95703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">

</xml_diff>

<commit_message>
add preliminary method "new_verba" (HACKY!!!): approach to - allow assigning of other dataset variables by verbatim data - keep the value labels - assign variable label like "mdg"
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="162">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -316,6 +316,9 @@
     <t xml:space="preserve">ex_further_cond</t>
   </si>
   <si>
+    <t xml:space="preserve">ex_assign</t>
+  </si>
+  <si>
     <t xml:space="preserve">Q6</t>
   </si>
   <si>
@@ -350,6 +353,12 @@
   </si>
   <si>
     <t xml:space="preserve">q6n{nn}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mdg_custom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q6mw_{nn}</t>
   </si>
   <si>
     <t xml:space="preserve">#COMP</t>
@@ -660,7 +669,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11.8046875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -750,7 +759,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.25390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -871,7 +880,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.25390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1251,8 +1260,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:S22"/>
-  <sheetFormatPr defaultColWidth="11.09375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="B1:T23"/>
+  <sheetFormatPr defaultColWidth="11.109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
@@ -1364,6 +1373,9 @@
       <c r="S17" s="1" t="s">
         <v>93</v>
       </c>
+      <c r="T17" s="0" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
@@ -1373,33 +1385,33 @@
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H18" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="R18" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="R18" s="1" t="s">
-        <v>94</v>
-      </c>
       <c r="S18" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H19" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="R19" s="1" t="s">
         <v>99</v>
-      </c>
-      <c r="R19" s="1" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1410,13 +1422,13 @@
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1427,19 +1439,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1456,13 +1468,30 @@
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="D23" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="T23" s="0" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1482,7 +1511,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="11.23828125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.25390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1498,50 +1527,50 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1555,7 +1584,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1574,7 +1603,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1586,15 +1615,15 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>29</v>
@@ -1602,7 +1631,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>43</v>
@@ -1613,24 +1642,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1638,7 +1667,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1646,23 +1675,23 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>43</v>
@@ -1670,61 +1699,61 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="5" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>30</v>
@@ -1735,70 +1764,70 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="6" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="6" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1820,7 +1849,7 @@
         <v>2</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1867,14 +1896,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.95703125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.9765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
- add "type" column to Excel mapping "Variables" sheet - add new function `update_var_sheet()`
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" state="visible" r:id="rId2"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="166">
   <si>
     <t xml:space="preserve">item</t>
   </si>
@@ -94,6 +94,9 @@
     <t xml:space="preserve">varlab</t>
   </si>
   <si>
+    <t xml:space="preserve">type</t>
+  </si>
+  <si>
     <t xml:space="preserve">new_label</t>
   </si>
   <si>
@@ -109,6 +112,9 @@
     <t xml:space="preserve">How much do you like the product?</t>
   </si>
   <si>
+    <t xml:space="preserve">double</t>
+  </si>
+  <si>
     <t xml:space="preserve">Like Product</t>
   </si>
   <si>
@@ -149,6 +155,12 @@
   </si>
   <si>
     <t xml:space="preserve">q6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tell me something positive.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">character</t>
   </si>
   <si>
     <t xml:space="preserve">a</t>
@@ -669,7 +681,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="11.82421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.8125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -745,7 +757,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
@@ -758,10 +770,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultColWidth="11.25390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
@@ -777,96 +789,126 @@
       <c r="E1" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C2" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" s="0" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="D3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>33</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>35</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>38</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>40</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C8" s="0" t="s">
         <v>42</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>46</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -880,43 +922,43 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="11.25390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -924,68 +966,68 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G6" s="1"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>1</v>
@@ -994,192 +1036,192 @@
         <v>6</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G23" s="1" t="n">
         <v>1</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B24" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G24" s="1" t="n">
         <v>1</v>
@@ -1187,47 +1229,47 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="G25" s="1" t="n">
         <v>2</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="G26" s="1" t="n">
         <v>3</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G27" s="1" t="n">
         <v>3</v>
@@ -1235,19 +1277,19 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B28" s="1" t="n">
         <v>99</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1261,53 +1303,53 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="B1:T23"/>
-  <sheetFormatPr defaultColWidth="11.109375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.1015625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="1" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="1" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>2</v>
@@ -1315,120 +1357,120 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="Q17" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="S17" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="T17" s="0" t="s">
-        <v>94</v>
+        <v>97</v>
+      </c>
+      <c r="T17" s="1" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="S18" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
       <c r="H20" s="3" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
@@ -1439,19 +1481,19 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="3" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
       <c r="G21" s="3"/>
       <c r="H21" s="3" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
@@ -1462,42 +1504,42 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C22" s="1" t="n">
         <v>2</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="L22" s="1" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="0" t="s">
-        <v>38</v>
-      </c>
-      <c r="C23" s="0" t="s">
-        <v>107</v>
-      </c>
-      <c r="D23" s="0" t="s">
-        <v>101</v>
+      <c r="B23" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="T23" s="0" t="s">
-        <v>23</v>
+        <v>112</v>
+      </c>
+      <c r="T23" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1511,7 +1553,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:F49"/>
-  <sheetFormatPr defaultColWidth="11.25390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.25" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1"/>
@@ -1527,50 +1569,50 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="F3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1584,7 +1626,7 @@
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1603,7 +1645,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>4</v>
@@ -1615,26 +1657,26 @@
         <v>3</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C13" s="1" t="n">
         <v>1</v>
@@ -1642,24 +1684,24 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1667,7 +1709,7 @@
         <v>1</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1675,159 +1717,159 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>3</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="5" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C28" s="5" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C33" s="6" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C34" s="6" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1838,7 +1880,7 @@
         <v>1</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1849,7 +1891,7 @@
         <v>2</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1881,8 +1923,8 @@
     <hyperlink ref="C34" r:id="rId1" display="see here: https://superuser.com/a/643521"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -1896,14 +1938,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:C2"/>
-  <sheetFormatPr defaultColWidth="11.9765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.96875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="C2" s="1" t="n">
         <v>3</v>
@@ -1912,7 +1954,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>

</xml_diff>

<commit_message>
delete rows after dot (".") in Free sheets
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B772BD6-E6B6-4E29-BDB2-ED53EE503079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E859DD-ECF9-49F0-8E90-9395C4523242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="17812" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="17812" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="171">
   <si>
     <t>item</t>
   </si>
@@ -556,6 +556,9 @@
   </si>
   <si>
     <t>q99</t>
+  </si>
+  <si>
+    <t>line should be reomoved! (below dot "." in first column…)</t>
   </si>
 </sst>
 </file>
@@ -565,7 +568,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -588,6 +591,13 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -622,7 +632,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -630,6 +640,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1859,7 +1870,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F49"/>
+  <dimension ref="A1:F50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
@@ -1967,251 +1978,271 @@
         <v>127</v>
       </c>
     </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="B11" s="1">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1">
+        <v>2</v>
+      </c>
+      <c r="D11" s="1">
+        <v>3</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>170</v>
+      </c>
+    </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A12" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>31</v>
+      <c r="B12" s="1">
+        <v>1</v>
+      </c>
+      <c r="C12" s="1">
+        <v>2</v>
+      </c>
+      <c r="D12" s="1">
+        <v>3</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A13" s="1" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="1">
-        <v>1</v>
+        <v>129</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.4">
       <c r="A14" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+      <c r="A15" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B15" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C15" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A16" s="1" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A17" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B17" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>134</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="B17" s="1">
-        <v>1</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="B18" s="1">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B19" s="1">
         <v>2</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C19" s="1" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A19" s="1" t="s">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A20" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B20" s="1">
         <v>3</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C20" s="1" t="s">
         <v>137</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A21" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A23" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B23" s="1">
         <v>4</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C23" s="1" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A26" s="1" t="s">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A27" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B27" s="1" t="s">
         <v>140</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C27" s="1" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="B27" s="5" t="s">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B28" s="5" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="C28" s="5" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="C29" s="5" t="s">
         <v>142</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A29" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A31" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B31" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C30" s="1" t="s">
+      <c r="C31" s="1" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A32" s="1" t="s">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A33" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B33" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C32" s="1" t="s">
+      <c r="C33" s="1" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="C33" s="6" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.4">
       <c r="C34" s="6" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="C35" s="6" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A35" s="1" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A36" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B36" s="1" t="s">
         <v>151</v>
       </c>
-      <c r="C35" s="1" t="s">
+      <c r="C36" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A37" s="1" t="s">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A38" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B38" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="C37" s="1" t="s">
+      <c r="C38" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D37" s="1" t="s">
+      <c r="D38" s="1" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A39" s="1" t="s">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A40" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B40" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="C39" s="1" t="s">
+      <c r="C40" s="1" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A41" s="1" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A42" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B42" s="1" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A44" s="1" t="s">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A45" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B45" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="C44" s="1" t="s">
+      <c r="C45" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="D44" s="1" t="s">
+      <c r="D45" s="1" t="s">
         <v>163</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="B45" s="1">
-        <v>1</v>
-      </c>
-      <c r="D45" s="1">
-        <v>1</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.4">
       <c r="B46" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D46" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>164</v>
+        <v>43</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.4">
       <c r="B47" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D47" s="1">
         <v>2</v>
       </c>
+      <c r="E47" s="1" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.4">
       <c r="B48" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D48" s="1">
         <v>2</v>
@@ -2219,15 +2250,23 @@
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.4">
       <c r="B49" s="1">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D49" s="1">
         <v>2</v>
       </c>
     </row>
+    <row r="50" spans="2:4" x14ac:dyDescent="0.4">
+      <c r="B50" s="1">
+        <v>5</v>
+      </c>
+      <c r="D50" s="1">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C34" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
+    <hyperlink ref="C35" r:id="rId1" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>

<commit_message>
add new command_block #RMVAL to: - remove values & - value labels of specified values
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8E859DD-ECF9-49F0-8E90-9395C4523242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1C226D4-CF23-48F9-BD5B-7764E7CDD2FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="17812" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="172">
   <si>
     <t>item</t>
   </si>
@@ -559,6 +559,9 @@
   </si>
   <si>
     <t>line should be reomoved! (below dot "." in first column…)</t>
+  </si>
+  <si>
+    <t>#RMVAL</t>
   </si>
 </sst>
 </file>
@@ -1870,7 +1873,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
@@ -2248,7 +2251,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
       <c r="B49" s="1">
         <v>4</v>
       </c>
@@ -2256,12 +2259,25 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.4">
       <c r="B50" s="1">
         <v>5</v>
       </c>
       <c r="D50" s="1">
         <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A53" t="s">
+        <v>171</v>
+      </c>
+      <c r="B53" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B54">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modify #RMVAL: - add possibility to assign result to new vector (if empty, original is modified) - add possibility to modify variable label (if empty, original is kept)
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1C226D4-CF23-48F9-BD5B-7764E7CDD2FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED8EACC5-218C-4CCE-B22A-C7E4CB0122D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="17812" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="267" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="173">
   <si>
     <t>item</t>
   </si>
@@ -562,6 +562,9 @@
   </si>
   <si>
     <t>#RMVAL</t>
+  </si>
+  <si>
+    <t>new_varlab</t>
   </si>
 </sst>
 </file>
@@ -2274,6 +2277,12 @@
       <c r="B53" t="s">
         <v>24</v>
       </c>
+      <c r="C53" t="s">
+        <v>24</v>
+      </c>
+      <c r="D53" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.4">
       <c r="B54">

</xml_diff>

<commit_message>
also adapt package mapping file to test for last commit (35baac39b5f26cffea570f470f6c9635cdac7c85)
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED8EACC5-218C-4CCE-B22A-C7E4CB0122D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F3CB3F-6C97-4E86-AE0F-598400139A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="17812" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -468,9 +468,6 @@
     <t>added label</t>
   </si>
   <si>
-    <t>q{3 5}</t>
-  </si>
-  <si>
     <t>Almost same variable label for q{3 5} and q{5 3}</t>
   </si>
   <si>
@@ -565,6 +562,9 @@
   </si>
   <si>
     <t>new_varlab</t>
+  </si>
+  <si>
+    <t>q{ 3 5}</t>
   </si>
 </sst>
 </file>
@@ -638,14 +638,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -965,73 +964,73 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5">
         <v>-2</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>16</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1051,61 +1050,61 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>25</v>
       </c>
       <c r="C2" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>29</v>
       </c>
       <c r="C3" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>33</v>
       </c>
       <c r="C4" t="s">
@@ -1113,35 +1112,35 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>35</v>
       </c>
       <c r="C5" t="s">
         <v>26</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>38</v>
       </c>
       <c r="C6" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>40</v>
       </c>
       <c r="B7" t="s">
@@ -1150,35 +1149,35 @@
       <c r="C7" t="s">
         <v>42</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>45</v>
       </c>
       <c r="C8" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" t="s">
         <v>46</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>48</v>
       </c>
       <c r="C9" t="s">
         <v>26</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" t="s">
         <v>49</v>
       </c>
     </row>
@@ -1194,364 +1193,355 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>21</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>53</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>54</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>56</v>
       </c>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3">
         <v>2</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>57</v>
       </c>
-      <c r="G3" s="1"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A4" s="1" t="s">
+      <c r="A4" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>58</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A5" s="1" t="s">
+      <c r="A5" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5">
         <v>4</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>59</v>
       </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A6" s="1" t="s">
+      <c r="A6" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6">
         <v>5</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>60</v>
       </c>
-      <c r="G6" s="1"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7">
         <v>99</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
         <v>28</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8">
         <v>1</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9">
         <v>2</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>28</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10">
         <v>99</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A11" s="1" t="s">
+      <c r="A11" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11">
         <v>1</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A12" s="1" t="s">
+      <c r="A12" t="s">
         <v>32</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12">
         <v>2</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13">
         <v>3</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14">
         <v>4</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15">
         <v>5</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A16" s="1" t="s">
+      <c r="A16" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16">
         <v>99</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17">
         <v>1</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A18" s="1" t="s">
+      <c r="A18" t="s">
         <v>34</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18">
         <v>2</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A19" s="1" t="s">
+      <c r="A19" t="s">
         <v>34</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19">
         <v>3</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>34</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20">
         <v>4</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A21" s="1" t="s">
+      <c r="A21" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21">
         <v>5</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A22" s="1" t="s">
+      <c r="A22" t="s">
         <v>34</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22">
         <v>99</v>
       </c>
-      <c r="C22" s="1" t="s">
+      <c r="C22" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A23" s="1" t="s">
+      <c r="A23" t="s">
         <v>37</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23">
         <v>1</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" t="s">
         <v>56</v>
       </c>
-      <c r="F23" s="1" t="s">
+      <c r="F23" t="s">
         <v>64</v>
       </c>
-      <c r="G23" s="1">
+      <c r="G23">
         <v>1</v>
       </c>
-      <c r="H23" s="1" t="s">
+      <c r="H23" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A24" s="1" t="s">
+      <c r="A24" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="1">
+      <c r="B24">
         <v>2</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" t="s">
         <v>57</v>
       </c>
-      <c r="G24" s="1">
+      <c r="G24">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A25" s="1" t="s">
+      <c r="A25" t="s">
         <v>37</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B25">
         <v>3</v>
       </c>
-      <c r="C25" s="1" t="s">
+      <c r="C25" t="s">
         <v>58</v>
       </c>
-      <c r="G25" s="1">
+      <c r="G25">
         <v>2</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="H25" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A26" s="1" t="s">
+      <c r="A26" t="s">
         <v>37</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26">
         <v>4</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C26" t="s">
         <v>59</v>
       </c>
-      <c r="G26" s="1">
+      <c r="G26">
         <v>3</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="H26" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A27" s="1" t="s">
+      <c r="A27" t="s">
         <v>37</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27">
         <v>5</v>
       </c>
-      <c r="C27" s="1" t="s">
+      <c r="C27" t="s">
         <v>60</v>
       </c>
-      <c r="G27" s="1">
+      <c r="G27">
         <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.4">
-      <c r="A28" s="1" t="s">
+      <c r="A28" t="s">
         <v>37</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B28">
         <v>99</v>
       </c>
-      <c r="C28" s="1" t="s">
+      <c r="C28" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1593,7 +1583,7 @@
         <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C5">
         <v>10</v>
@@ -1604,7 +1594,7 @@
         <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C6">
         <v>11</v>
@@ -1621,251 +1611,251 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>70</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>76</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>78</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.4">
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="17" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>80</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>81</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" t="s">
         <v>82</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" t="s">
         <v>83</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F17" t="s">
         <v>84</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="G17" t="s">
         <v>85</v>
       </c>
-      <c r="H17" s="1" t="s">
+      <c r="H17" t="s">
         <v>86</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="I17" t="s">
         <v>87</v>
       </c>
-      <c r="J17" s="1" t="s">
+      <c r="J17" t="s">
         <v>88</v>
       </c>
-      <c r="K17" s="1" t="s">
+      <c r="K17" t="s">
         <v>89</v>
       </c>
-      <c r="L17" s="1" t="s">
+      <c r="L17" t="s">
         <v>90</v>
       </c>
-      <c r="M17" s="1" t="s">
+      <c r="M17" t="s">
         <v>91</v>
       </c>
-      <c r="N17" s="1" t="s">
+      <c r="N17" t="s">
         <v>92</v>
       </c>
-      <c r="O17" s="1" t="s">
+      <c r="O17" t="s">
         <v>93</v>
       </c>
-      <c r="P17" s="1" t="s">
+      <c r="P17" t="s">
         <v>94</v>
       </c>
-      <c r="Q17" s="1" t="s">
+      <c r="Q17" t="s">
         <v>95</v>
       </c>
-      <c r="R17" s="1" t="s">
+      <c r="R17" t="s">
         <v>96</v>
       </c>
-      <c r="S17" s="1" t="s">
+      <c r="S17" t="s">
         <v>97</v>
       </c>
-      <c r="T17" s="1" t="s">
+      <c r="T17" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="18" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>40</v>
       </c>
-      <c r="C18" s="1">
+      <c r="C18">
         <v>1</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" t="s">
         <v>99</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="H18" t="s">
         <v>100</v>
       </c>
-      <c r="R18" s="1" t="s">
+      <c r="R18" t="s">
         <v>99</v>
       </c>
-      <c r="S18" s="1" t="s">
+      <c r="S18" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="19" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>102</v>
       </c>
-      <c r="C19" s="1">
+      <c r="C19">
         <v>1</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" t="s">
         <v>103</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="H19" t="s">
         <v>104</v>
       </c>
-      <c r="R19" s="1" t="s">
+      <c r="R19" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="20" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="2">
         <v>3</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="D20" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3" t="s">
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3">
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2">
         <v>100</v>
       </c>
     </row>
     <row r="21" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="2">
         <v>3</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="D21" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3" t="s">
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3">
+      <c r="I21" s="2"/>
+      <c r="J21" s="2"/>
+      <c r="K21" s="2"/>
+      <c r="L21" s="2">
         <v>100</v>
       </c>
     </row>
     <row r="22" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>40</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22">
         <v>2</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" t="s">
         <v>109</v>
       </c>
-      <c r="H22" s="1" t="s">
+      <c r="H22" t="s">
         <v>110</v>
       </c>
-      <c r="L22" s="1">
+      <c r="L22">
         <v>100</v>
       </c>
     </row>
     <row r="23" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B23" s="1" t="s">
+      <c r="B23" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" t="s">
         <v>111</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" t="s">
         <v>105</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="H23" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="T23" s="1" t="s">
+      <c r="T23" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.4">
-      <c r="B24" s="1" t="s">
+      <c r="B24" t="s">
         <v>40</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="C24" t="s">
         <v>111</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" t="s">
         <v>105</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="H24" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="T24" t="s">
         <v>166</v>
-      </c>
-      <c r="T24" s="1" t="s">
-        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -1880,399 +1870,393 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="F1" s="4"/>
+      <c r="F1" s="3"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="F2" s="4"/>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
         <v>113</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>115</v>
       </c>
-      <c r="F3" s="4"/>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A7" s="1" t="s">
+      <c r="A7" t="s">
         <v>121</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>122</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>123</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="B8" s="1">
+      <c r="B8">
         <v>1</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8">
         <v>2</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8">
         <v>1</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="B9" s="1">
+      <c r="B9">
         <v>3</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9">
         <v>3</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9">
         <v>2</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9">
         <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A10" s="1" t="s">
+      <c r="A10" t="s">
         <v>126</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10">
         <v>4</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10">
         <v>5</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10">
         <v>3</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="B11" s="1">
+      <c r="B11">
         <v>1</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11">
         <v>2</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11">
         <v>3</v>
       </c>
-      <c r="E11" s="7" t="s">
-        <v>170</v>
+      <c r="E11" s="6" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="B12" s="1">
+      <c r="B12">
         <v>1</v>
       </c>
-      <c r="C12" s="1">
+      <c r="C12">
         <v>2</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12">
         <v>3</v>
       </c>
-      <c r="E12" s="7" t="s">
-        <v>170</v>
+      <c r="E12" s="6" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A13" s="1" t="s">
+      <c r="A13" t="s">
         <v>128</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>129</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A14" s="1" t="s">
+      <c r="A14" t="s">
         <v>113</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.4">
-      <c r="A15" s="1" t="s">
+      <c r="A15" t="s">
         <v>130</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>131</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A17" s="1" t="s">
+      <c r="A17" t="s">
         <v>133</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="B18" s="1">
+      <c r="B18">
         <v>1</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="B19" s="1">
+      <c r="B19">
         <v>2</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A20" s="1" t="s">
+      <c r="A20" t="s">
         <v>126</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20">
         <v>3</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A22" s="1" t="s">
+      <c r="A22" t="s">
         <v>138</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A23" s="1" t="s">
+      <c r="A23" t="s">
         <v>126</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23">
         <v>4</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A27" s="1" t="s">
+      <c r="A27" t="s">
         <v>130</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" t="s">
+        <v>172</v>
+      </c>
+      <c r="C27" t="s">
         <v>140</v>
       </c>
-      <c r="C27" s="1" t="s">
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="B28" s="4" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="B28" s="5" t="s">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="C29" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>113</v>
+      </c>
+      <c r="B30" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="C29" s="5" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A30" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B30" s="1" t="s">
+      <c r="C30" t="s">
         <v>143</v>
       </c>
-      <c r="C30" s="1" t="s">
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>130</v>
+      </c>
+      <c r="B31" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A31" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="B31" s="1" t="s">
+      <c r="C31" t="s">
         <v>145</v>
       </c>
-      <c r="C31" s="1" t="s">
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A33" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A33" s="1" t="s">
+      <c r="B33" t="s">
+        <v>32</v>
+      </c>
+      <c r="C33" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="C34" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="B33" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="C34" s="6" t="s">
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="C35" s="5" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="C35" s="6" t="s">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A36" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A36" s="1" t="s">
+      <c r="B36" t="s">
         <v>150</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="C36" t="s">
         <v>151</v>
       </c>
-      <c r="C36" s="1" t="s">
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A38" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A38" s="1" t="s">
+      <c r="B38" t="s">
         <v>153</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="C38" t="s">
+        <v>4</v>
+      </c>
+      <c r="D38" t="s">
         <v>154</v>
       </c>
-      <c r="C38" s="1" t="s">
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A40" t="s">
+        <v>155</v>
+      </c>
+      <c r="B40" t="s">
+        <v>156</v>
+      </c>
+      <c r="C40" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A42" t="s">
+        <v>158</v>
+      </c>
+      <c r="B42" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A45" t="s">
+        <v>121</v>
+      </c>
+      <c r="B45" t="s">
+        <v>160</v>
+      </c>
+      <c r="C45" t="s">
+        <v>161</v>
+      </c>
+      <c r="D45" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="B46">
+        <v>1</v>
+      </c>
+      <c r="D46">
+        <v>1</v>
+      </c>
+      <c r="E46" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="B47">
+        <v>2</v>
+      </c>
+      <c r="D47">
+        <v>2</v>
+      </c>
+      <c r="E47" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="B48">
+        <v>3</v>
+      </c>
+      <c r="D48">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="B49">
         <v>4</v>
       </c>
-      <c r="D38" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A40" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A42" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A45" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="B46" s="1">
-        <v>1</v>
-      </c>
-      <c r="D46" s="1">
-        <v>1</v>
-      </c>
-      <c r="E46" s="1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="B47" s="1">
+      <c r="D49">
         <v>2</v>
       </c>
-      <c r="D47" s="1">
-        <v>2</v>
-      </c>
-      <c r="E47" s="1" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="B48" s="1">
-        <v>3</v>
-      </c>
-      <c r="D48" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="B49" s="1">
-        <v>4</v>
-      </c>
-      <c r="D49" s="1">
-        <v>2</v>
-      </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="B50" s="1">
+      <c r="B50">
         <v>5</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50">
         <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A53" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B53" t="s">
         <v>24</v>
@@ -2281,7 +2265,7 @@
         <v>24</v>
       </c>
       <c r="D53" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.4">
@@ -2304,13 +2288,13 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="2" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>113</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="C2" s="1">
+      <c r="B2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C2">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
breaking change: - The #R command now can be passed multiple lines of arbitrary R code in column B - the command has been removed from the test via the mapping file in inst/extdata/mapping.xlsx (because the test from Rstudio the build pane doesn't work, but the from command line it works :(  ...) - the commands now are evaluated in the environment from where the R Mapping R6 object is generated (I think that's the reason why it doesn't work in the test from the build pane)
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F3CB3F-6C97-4E86-AE0F-598400139A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8973239-436A-42B7-8BB6-F6776DFEB4FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="17812" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="178">
   <si>
     <t>item</t>
   </si>
@@ -525,9 +525,6 @@
     <t xml:space="preserve">#R </t>
   </si>
   <si>
-    <t>data.frame(a=1)</t>
-  </si>
-  <si>
     <t xml:space="preserve">q1  </t>
   </si>
   <si>
@@ -565,6 +562,24 @@
   </si>
   <si>
     <t>q{ 3 5}</t>
+  </si>
+  <si>
+    <t>xyz1 &lt;- haven::labelled(xyz0, labels = c(efg = 3), label = "varlab xyz")</t>
+  </si>
+  <si>
+    <t>xyz0 &lt;- 8 - 6 + 1</t>
+  </si>
+  <si>
+    <t>m$dat_mod$xyz &lt;- xyz1</t>
+  </si>
+  <si>
+    <t>m$dat_mod$xyz &lt;- NULL</t>
+  </si>
+  <si>
+    <t>m$dat_mod$a &lt;- 1</t>
+  </si>
+  <si>
+    <t>test from Rstudio build pane doesn't work, but from command line it works :(</t>
   </si>
 </sst>
 </file>
@@ -606,7 +621,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -625,6 +640,12 @@
         <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -638,7 +659,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -646,6 +667,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1583,7 +1605,7 @@
         <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C5">
         <v>10</v>
@@ -1594,7 +1616,7 @@
         <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C6">
         <v>11</v>
@@ -1852,10 +1874,10 @@
         <v>105</v>
       </c>
       <c r="H24" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="T24" t="s">
         <v>165</v>
-      </c>
-      <c r="T24" t="s">
-        <v>166</v>
       </c>
     </row>
   </sheetData>
@@ -1866,7 +1888,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.4">
@@ -1979,7 +2001,7 @@
         <v>3</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.4">
@@ -1993,7 +2015,7 @@
         <v>3</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.4">
@@ -2091,7 +2113,7 @@
         <v>130</v>
       </c>
       <c r="B27" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C27" t="s">
         <v>140</v>
@@ -2129,7 +2151,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A33" t="s">
         <v>146</v>
       </c>
@@ -2140,17 +2162,17 @@
         <v>36</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
       <c r="C34" s="5" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
       <c r="C35" s="5" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A36" t="s">
         <v>149</v>
       </c>
@@ -2161,7 +2183,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>152</v>
       </c>
@@ -2175,7 +2197,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
       <c r="A40" t="s">
         <v>155</v>
       </c>
@@ -2186,90 +2208,119 @@
         <v>157</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A42" t="s">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="F41" s="7" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="F42" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="B42" t="s">
+      <c r="G42" s="7" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="F43" s="7"/>
+      <c r="G43" s="7" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="F44" s="7"/>
+      <c r="G44" s="7" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="F45" s="7"/>
+      <c r="G45" s="7" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="F46" s="7"/>
+      <c r="G46" s="7" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.4">
+      <c r="A48" t="s">
+        <v>121</v>
+      </c>
+      <c r="B48" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A45" t="s">
-        <v>121</v>
-      </c>
-      <c r="B45" t="s">
+      <c r="C48" t="s">
         <v>160</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D48" t="s">
         <v>161</v>
       </c>
-      <c r="D45" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="B46">
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="B49">
         <v>1</v>
       </c>
-      <c r="D46">
+      <c r="D49">
         <v>1</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E49" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="B47">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="B50">
         <v>2</v>
-      </c>
-      <c r="D47">
-        <v>2</v>
-      </c>
-      <c r="E47" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="B48">
-        <v>3</v>
-      </c>
-      <c r="D48">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="B49">
-        <v>4</v>
-      </c>
-      <c r="D49">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="B50">
-        <v>5</v>
       </c>
       <c r="D50">
         <v>2</v>
       </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A53" t="s">
+      <c r="E50" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="B51">
+        <v>3</v>
+      </c>
+      <c r="D51">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="B52">
+        <v>4</v>
+      </c>
+      <c r="D52">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="B53">
+        <v>5</v>
+      </c>
+      <c r="D53">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A56" t="s">
+        <v>169</v>
+      </c>
+      <c r="B56" t="s">
+        <v>24</v>
+      </c>
+      <c r="C56" t="s">
+        <v>24</v>
+      </c>
+      <c r="D56" t="s">
         <v>170</v>
       </c>
-      <c r="B53" t="s">
-        <v>24</v>
-      </c>
-      <c r="C53" t="s">
-        <v>24</v>
-      </c>
-      <c r="D53" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="B54">
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="B57">
         <v>99</v>
       </c>
     </row>
@@ -2292,7 +2343,7 @@
         <v>113</v>
       </c>
       <c r="B2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C2">
         <v>3</v>

</xml_diff>

<commit_message>
add new command block: - #RENAME for Free sheets - with class cmd_rename
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8973239-436A-42B7-8BB6-F6776DFEB4FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719D0518-BA65-40B6-BB1E-D95681F33F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="17812" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="14250" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="configr" sheetId="1" r:id="rId1"/>
@@ -30,14 +30,6 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -46,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="181">
   <si>
     <t>item</t>
   </si>
@@ -580,6 +572,15 @@
   </si>
   <si>
     <t>test from Rstudio build pane doesn't work, but from command line it works :(</t>
+  </si>
+  <si>
+    <t>#RENAME</t>
+  </si>
+  <si>
+    <t>q2new</t>
+  </si>
+  <si>
+    <t>q4new</t>
   </si>
 </sst>
 </file>
@@ -974,7 +975,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme 2013 - 2022" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -983,9 +984,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.84375" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -996,7 +997,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1004,7 +1005,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -1015,7 +1016,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -1026,7 +1027,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -1037,7 +1038,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>13</v>
       </c>
@@ -1045,7 +1046,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>15</v>
       </c>
@@ -1069,9 +1070,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -1091,7 +1092,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -1105,7 +1106,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -1122,7 +1123,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -1133,7 +1134,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>34</v>
       </c>
@@ -1147,7 +1148,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -1161,7 +1162,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>40</v>
       </c>
@@ -1175,7 +1176,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>44</v>
       </c>
@@ -1192,7 +1193,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>48</v>
       </c>
@@ -1212,9 +1213,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -1240,7 +1241,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -1251,7 +1252,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -1262,7 +1263,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>24</v>
       </c>
@@ -1273,7 +1274,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1284,7 +1285,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>24</v>
       </c>
@@ -1295,7 +1296,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -1306,7 +1307,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -1320,7 +1321,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -1331,7 +1332,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>28</v>
       </c>
@@ -1342,7 +1343,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>32</v>
       </c>
@@ -1353,7 +1354,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>32</v>
       </c>
@@ -1364,7 +1365,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -1375,7 +1376,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>32</v>
       </c>
@@ -1386,7 +1387,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -1397,7 +1398,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -1408,7 +1409,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>34</v>
       </c>
@@ -1419,7 +1420,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>34</v>
       </c>
@@ -1430,7 +1431,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>34</v>
       </c>
@@ -1441,7 +1442,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>34</v>
       </c>
@@ -1452,7 +1453,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>34</v>
       </c>
@@ -1463,7 +1464,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>34</v>
       </c>
@@ -1474,7 +1475,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>37</v>
       </c>
@@ -1494,7 +1495,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1508,7 +1509,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>37</v>
       </c>
@@ -1525,7 +1526,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>37</v>
       </c>
@@ -1542,7 +1543,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -1556,7 +1557,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>37</v>
       </c>
@@ -1576,9 +1577,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CCDC469-55AD-4BDB-AD79-F77691D63E27}">
   <dimension ref="A3:C6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>113</v>
       </c>
@@ -1589,7 +1590,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>113</v>
       </c>
@@ -1600,7 +1601,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>113</v>
       </c>
@@ -1611,7 +1612,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>113</v>
       </c>
@@ -1630,9 +1631,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B1:T24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.07421875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
         <v>68</v>
       </c>
@@ -1640,7 +1641,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>70</v>
       </c>
@@ -1648,17 +1649,17 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>74</v>
       </c>
@@ -1666,7 +1667,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>76</v>
       </c>
@@ -1674,7 +1675,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>78</v>
       </c>
@@ -1682,12 +1683,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="17" spans="2:20" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>80</v>
       </c>
@@ -1746,7 +1747,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="18" spans="2:20" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>40</v>
       </c>
@@ -1766,7 +1767,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="19" spans="2:20" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>102</v>
       </c>
@@ -1783,7 +1784,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="20" spans="2:20" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
         <v>40</v>
       </c>
@@ -1806,7 +1807,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="2:20" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>107</v>
       </c>
@@ -1829,7 +1830,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="22" spans="2:20" x14ac:dyDescent="0.4">
+    <row r="22" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>40</v>
       </c>
@@ -1846,7 +1847,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="23" spans="2:20" x14ac:dyDescent="0.4">
+    <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>40</v>
       </c>
@@ -1863,7 +1864,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="24" spans="2:20" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>40</v>
       </c>
@@ -1888,16 +1889,16 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.23046875" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:G60"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F1" s="3"/>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>113</v>
       </c>
@@ -1909,7 +1910,7 @@
       </c>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>116</v>
       </c>
@@ -1920,7 +1921,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>116</v>
       </c>
@@ -1931,7 +1932,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>121</v>
       </c>
@@ -1945,7 +1946,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B8">
         <v>1</v>
       </c>
@@ -1959,7 +1960,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B9">
         <v>3</v>
       </c>
@@ -1973,7 +1974,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>126</v>
       </c>
@@ -1990,7 +1991,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B11">
         <v>1</v>
       </c>
@@ -2004,7 +2005,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="B12">
         <v>1</v>
       </c>
@@ -2018,7 +2019,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>128</v>
       </c>
@@ -2029,7 +2030,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>113</v>
       </c>
@@ -2040,7 +2041,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>130</v>
       </c>
@@ -2051,7 +2052,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>133</v>
       </c>
@@ -2062,7 +2063,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B18">
         <v>1</v>
       </c>
@@ -2070,7 +2071,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B19">
         <v>2</v>
       </c>
@@ -2078,7 +2079,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>126</v>
       </c>
@@ -2089,7 +2090,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>138</v>
       </c>
@@ -2097,7 +2098,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>126</v>
       </c>
@@ -2108,7 +2109,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>130</v>
       </c>
@@ -2119,17 +2120,17 @@
         <v>140</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="B28" s="4" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="C29" s="4" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>113</v>
       </c>
@@ -2140,7 +2141,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>130</v>
       </c>
@@ -2151,7 +2152,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>146</v>
       </c>
@@ -2162,17 +2163,17 @@
         <v>36</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C34" s="5" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="C35" s="5" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>149</v>
       </c>
@@ -2183,7 +2184,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>152</v>
       </c>
@@ -2197,7 +2198,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>155</v>
       </c>
@@ -2208,12 +2209,12 @@
         <v>157</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F41" s="7" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F42" s="7" t="s">
         <v>158</v>
       </c>
@@ -2221,31 +2222,31 @@
         <v>173</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F43" s="7"/>
       <c r="G43" s="7" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F44" s="7"/>
       <c r="G44" s="7" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F45" s="7"/>
       <c r="G45" s="7" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F46" s="7"/>
       <c r="G46" s="7" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>121</v>
       </c>
@@ -2259,7 +2260,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B49">
         <v>1</v>
       </c>
@@ -2270,7 +2271,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B50">
         <v>2</v>
       </c>
@@ -2281,7 +2282,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B51">
         <v>3</v>
       </c>
@@ -2289,7 +2290,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B52">
         <v>4</v>
       </c>
@@ -2297,7 +2298,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B53">
         <v>5</v>
       </c>
@@ -2305,7 +2306,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>169</v>
       </c>
@@ -2319,9 +2320,28 @@
         <v>170</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B57">
         <v>99</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>178</v>
+      </c>
+      <c r="B59" t="s">
+        <v>31</v>
+      </c>
+      <c r="C59" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
+        <v>36</v>
+      </c>
+      <c r="C60" t="s">
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -2336,9 +2356,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A2:C2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>113</v>
       </c>

</xml_diff>

<commit_message>
add new Free sheet command block `#SELECT` (which passes the strings in column B as expressions to `dplyr::select()`
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{719D0518-BA65-40B6-BB1E-D95681F33F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4836679-E594-45A9-AD96-0E1C3246A623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="14250" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="185">
   <si>
     <t>item</t>
   </si>
@@ -581,6 +581,18 @@
   </si>
   <si>
     <t>q4new</t>
+  </si>
+  <si>
+    <t>#SELECT</t>
+  </si>
+  <si>
+    <t>-q4new</t>
+  </si>
+  <si>
+    <t>everything()</t>
+  </si>
+  <si>
+    <t>q2new:q3</t>
   </si>
 </sst>
 </file>
@@ -660,7 +672,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -669,6 +681,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -1889,7 +1902,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2343,6 +2356,27 @@
       <c r="C60" t="s">
         <v>180</v>
       </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>181</v>
+      </c>
+      <c r="B62" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B63" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B64" s="8" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B65" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
add new Free sheet command block `#FILTER` (which passes the strings in column B as expressions to `dplyr::filter()`
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4836679-E594-45A9-AD96-0E1C3246A623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C9AB776-6290-4B38-AA82-364F19728A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="14250" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="188">
   <si>
     <t>item</t>
   </si>
@@ -593,6 +593,15 @@
   </si>
   <si>
     <t>q2new:q3</t>
+  </si>
+  <si>
+    <t>#FILTER</t>
+  </si>
+  <si>
+    <t>!id %in% 21:100</t>
+  </si>
+  <si>
+    <t>!id %in% 10:19</t>
   </si>
 </sst>
 </file>
@@ -1902,7 +1911,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G65"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -2375,8 +2384,21 @@
         <v>182</v>
       </c>
     </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B65" s="8"/>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>185</v>
+      </c>
+      <c r="B66" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>187</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
remove #COMPR command block
</commit_message>
<xml_diff>
--- a/inst/extdata/mapping.xlsx
+++ b/inst/extdata/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\Projects\UW git\datenanpassr\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C9AB776-6290-4B38-AA82-364F19728A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92624FF8-811D-4BF0-9B25-81D8C847414A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="14250" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="187">
   <si>
     <t>item</t>
   </si>
@@ -485,9 +485,6 @@
   </si>
   <si>
     <t>see here: https://superuser.com/a/643521</t>
-  </si>
-  <si>
-    <t>#COMPR</t>
   </si>
   <si>
     <t>r_expr_var</t>
@@ -1628,7 +1625,7 @@
         <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C5">
         <v>10</v>
@@ -1639,7 +1636,7 @@
         <v>113</v>
       </c>
       <c r="B6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C6">
         <v>11</v>
@@ -1897,10 +1894,10 @@
         <v>105</v>
       </c>
       <c r="H24" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="T24" t="s">
         <v>164</v>
-      </c>
-      <c r="T24" t="s">
-        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -2024,7 +2021,7 @@
         <v>3</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -2038,7 +2035,7 @@
         <v>3</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -2136,7 +2133,7 @@
         <v>130</v>
       </c>
       <c r="B27" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C27" t="s">
         <v>140</v>
@@ -2197,75 +2194,75 @@
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
+        <v>113</v>
+      </c>
+      <c r="B36" t="s">
         <v>149</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>150</v>
-      </c>
-      <c r="C36" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>151</v>
+      </c>
+      <c r="B38" t="s">
         <v>152</v>
-      </c>
-      <c r="B38" t="s">
-        <v>153</v>
       </c>
       <c r="C38" t="s">
         <v>4</v>
       </c>
       <c r="D38" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
+        <v>154</v>
+      </c>
+      <c r="B40" t="s">
         <v>155</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>156</v>
-      </c>
-      <c r="C40" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F41" s="7" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F42" s="7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G42" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F43" s="7"/>
       <c r="G43" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F44" s="7"/>
       <c r="G44" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F45" s="7"/>
       <c r="G45" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="F46" s="7"/>
       <c r="G46" s="7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
@@ -2273,13 +2270,13 @@
         <v>121</v>
       </c>
       <c r="B48" t="s">
+        <v>158</v>
+      </c>
+      <c r="C48" t="s">
         <v>159</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>160</v>
-      </c>
-      <c r="D48" t="s">
-        <v>161</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -2301,7 +2298,7 @@
         <v>2</v>
       </c>
       <c r="E50" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
@@ -2330,7 +2327,7 @@
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B56" t="s">
         <v>24</v>
@@ -2339,7 +2336,7 @@
         <v>24</v>
       </c>
       <c r="D56" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -2349,13 +2346,13 @@
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B59" t="s">
         <v>31</v>
       </c>
       <c r="C59" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -2363,25 +2360,25 @@
         <v>36</v>
       </c>
       <c r="C60" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B62" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B64" s="8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.25">
@@ -2389,15 +2386,15 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>184</v>
+      </c>
+      <c r="B66" t="s">
         <v>185</v>
-      </c>
-      <c r="B66" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
   </sheetData>
@@ -2419,7 +2416,7 @@
         <v>113</v>
       </c>
       <c r="B2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C2">
         <v>3</v>

</xml_diff>